<commit_message>
changes in faculty unavailability
- instead of full day unavailablility, now specific timeslots can be selected for faculty unavailability
- verified with Q2 and Q5 scheduling, import-export working correctly with new changes
- documented the changes

TODOs:
- currently only section/area wise timetable is displayed, we can show course/faculty wise timetable, with seperate export functionality
- currently only single quarter can be scheduled at a time. expand it to schedule multiple quarters/years together
</commit_message>
<xml_diff>
--- a/static/Areas_timetable_config.xlsx
+++ b/static/Areas_timetable_config.xlsx
@@ -420,7 +420,7 @@
         <v>Exported at</v>
       </c>
       <c r="B2" t="str">
-        <v>5/27/2026, 6:22:07 PM</v>
+        <v>6/6/2026, 9:40:08 PM</v>
       </c>
     </row>
     <row r="3">
@@ -1739,7 +1739,7 @@
         <v>Max Load Per Day</v>
       </c>
       <c r="D1" t="str">
-        <v>Unavailable Dates (YYYY-MM-DD)</v>
+        <v>Unavailable Slots (YYYY-MM-DD|HH:MM-HH:MM;...)</v>
       </c>
     </row>
     <row r="2">
@@ -1851,7 +1851,7 @@
         <v>2</v>
       </c>
       <c r="D9" t="str">
-        <v/>
+        <v>2024-12-15|09:00-11:45; 2025-03-23|09:00-11:45</v>
       </c>
     </row>
     <row r="10">
@@ -1865,7 +1865,7 @@
         <v>2</v>
       </c>
       <c r="D10" t="str">
-        <v/>
+        <v>2025-01-10|19:00-21:45</v>
       </c>
     </row>
     <row r="11">
@@ -1907,7 +1907,7 @@
         <v>2</v>
       </c>
       <c r="D13" t="str">
-        <v/>
+        <v>2025-03-02|15:30-18:15</v>
       </c>
     </row>
     <row r="14">
@@ -1921,7 +1921,7 @@
         <v>2</v>
       </c>
       <c r="D14" t="str">
-        <v/>
+        <v>2025-03-23|15:30-18:15</v>
       </c>
     </row>
     <row r="15">
@@ -1963,7 +1963,7 @@
         <v>2</v>
       </c>
       <c r="D17" t="str">
-        <v/>
+        <v>2024-12-09|15:30-18:15</v>
       </c>
     </row>
     <row r="18">
@@ -1991,7 +1991,7 @@
         <v>2</v>
       </c>
       <c r="D19" t="str">
-        <v/>
+        <v>2025-01-13|15:30-18:15</v>
       </c>
     </row>
     <row r="20">
@@ -2005,7 +2005,7 @@
         <v>2</v>
       </c>
       <c r="D20" t="str">
-        <v/>
+        <v>2025-02-10|15:30-18:15</v>
       </c>
     </row>
     <row r="21">
@@ -2526,7 +2526,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L124"/>
+  <dimension ref="A1:L131"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2594,7 +2594,7 @@
         <v>11:45</v>
       </c>
       <c r="E2" t="str">
-        <v>SCM-A (ASS) / SCM-B (SSP) / SCM-C (RK)</v>
+        <v/>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -2603,7 +2603,7 @@
         <v/>
       </c>
       <c r="H2" t="str">
-        <v>ACCTP (DS)</v>
+        <v>DPI (SAA)</v>
       </c>
       <c r="I2" t="str">
         <v/>
@@ -2626,10 +2626,10 @@
         <v>Sunday</v>
       </c>
       <c r="C3" t="str">
-        <v>12:15</v>
+        <v>15:30</v>
       </c>
       <c r="D3" t="str">
-        <v>15:00</v>
+        <v>18:15</v>
       </c>
       <c r="E3" t="str">
         <v/>
@@ -2644,24 +2644,24 @@
         <v/>
       </c>
       <c r="I3" t="str">
-        <v/>
+        <v>AIB-B (VK)</v>
       </c>
       <c r="J3" t="str">
-        <v/>
+        <v>UOSWTPB (PS)</v>
       </c>
       <c r="K3" t="str">
         <v/>
       </c>
       <c r="L3" t="str">
-        <v>SI-B (PV) / MASA (KKS)</v>
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2024-12-01</v>
+        <v>2024-12-02</v>
       </c>
       <c r="B4" t="str">
-        <v>Sunday</v>
+        <v>Monday</v>
       </c>
       <c r="C4" t="str">
         <v>15:30</v>
@@ -2685,7 +2685,7 @@
         <v/>
       </c>
       <c r="J4" t="str">
-        <v>PBM-A (JJ)</v>
+        <v>PBM-B (SS)</v>
       </c>
       <c r="K4" t="str">
         <v/>
@@ -2696,16 +2696,16 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2024-12-02</v>
+        <v>2024-12-03</v>
       </c>
       <c r="B5" t="str">
-        <v>Monday</v>
+        <v>Tuesday</v>
       </c>
       <c r="C5" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D5" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E5" t="str">
         <v/>
@@ -2720,10 +2720,10 @@
         <v/>
       </c>
       <c r="I5" t="str">
-        <v/>
+        <v>AIB-A (MPS) / CSP (SRA)</v>
       </c>
       <c r="J5" t="str">
-        <v>MBM (JT) / MMT (PN)</v>
+        <v/>
       </c>
       <c r="K5" t="str">
         <v/>
@@ -2734,10 +2734,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2024-12-03</v>
+        <v>2024-12-04</v>
       </c>
       <c r="B6" t="str">
-        <v>Tuesday</v>
+        <v>Wednesday</v>
       </c>
       <c r="C6" t="str">
         <v>19:00</v>
@@ -2752,13 +2752,13 @@
         <v/>
       </c>
       <c r="G6" t="str">
-        <v/>
+        <v>AMA (PKB) / SAPM-A (ST) / SAPM-B (VB)</v>
       </c>
       <c r="H6" t="str">
         <v/>
       </c>
       <c r="I6" t="str">
-        <v>AIB-A (MPS) / CSP (SRA)</v>
+        <v/>
       </c>
       <c r="J6" t="str">
         <v/>
@@ -2772,10 +2772,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2024-12-04</v>
+        <v>2024-12-05</v>
       </c>
       <c r="B7" t="str">
-        <v>Wednesday</v>
+        <v>Thursday</v>
       </c>
       <c r="C7" t="str">
         <v>19:00</v>
@@ -2787,10 +2787,10 @@
         <v/>
       </c>
       <c r="F7" t="str">
-        <v/>
+        <v>IPP (SRN)</v>
       </c>
       <c r="G7" t="str">
-        <v>SAPM-B (VB) / PF (PKB) / ACF (ARS)</v>
+        <v/>
       </c>
       <c r="H7" t="str">
         <v/>
@@ -2805,15 +2805,15 @@
         <v/>
       </c>
       <c r="L7" t="str">
-        <v/>
+        <v>SI-B (PV) / MASA (KKS)</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2024-12-05</v>
+        <v>2024-12-06</v>
       </c>
       <c r="B8" t="str">
-        <v>Thursday</v>
+        <v>Friday</v>
       </c>
       <c r="C8" t="str">
         <v>19:00</v>
@@ -2822,10 +2822,10 @@
         <v>21:45</v>
       </c>
       <c r="E8" t="str">
-        <v/>
+        <v>SCM-A (ASS) / LSS-B (SG)</v>
       </c>
       <c r="F8" t="str">
-        <v>IPP (SRN)</v>
+        <v/>
       </c>
       <c r="G8" t="str">
         <v/>
@@ -2843,15 +2843,15 @@
         <v/>
       </c>
       <c r="L8" t="str">
-        <v>MTI-A (PV) / MTI-B (AK)</v>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2024-12-06</v>
+        <v>2024-12-07</v>
       </c>
       <c r="B9" t="str">
-        <v>Friday</v>
+        <v>Saturday</v>
       </c>
       <c r="C9" t="str">
         <v>19:00</v>
@@ -2860,16 +2860,16 @@
         <v>21:45</v>
       </c>
       <c r="E9" t="str">
-        <v>SCM-C (RK) / LSS-B (SG)</v>
+        <v/>
       </c>
       <c r="F9" t="str">
         <v/>
       </c>
       <c r="G9" t="str">
-        <v/>
+        <v>AMA (PKB) / SAPM-A (ST) / SAPM-B (VB)</v>
       </c>
       <c r="H9" t="str">
-        <v>ACCTP (DS) / DPI (SAA)</v>
+        <v/>
       </c>
       <c r="I9" t="str">
         <v/>
@@ -2886,19 +2886,19 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2024-12-07</v>
+        <v>2024-12-08</v>
       </c>
       <c r="B10" t="str">
-        <v>Saturday</v>
+        <v>Sunday</v>
       </c>
       <c r="C10" t="str">
-        <v>15:30</v>
+        <v>09:00</v>
       </c>
       <c r="D10" t="str">
-        <v>18:15</v>
+        <v>11:45</v>
       </c>
       <c r="E10" t="str">
-        <v/>
+        <v>SCM-A (ASS) / LSS-B (SG)</v>
       </c>
       <c r="F10" t="str">
         <v/>
@@ -2916,7 +2916,7 @@
         <v/>
       </c>
       <c r="K10" t="str">
-        <v>LSO (PNR)</v>
+        <v/>
       </c>
       <c r="L10" t="str">
         <v/>
@@ -2924,25 +2924,25 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2024-12-07</v>
+        <v>2024-12-08</v>
       </c>
       <c r="B11" t="str">
-        <v>Saturday</v>
+        <v>Sunday</v>
       </c>
       <c r="C11" t="str">
-        <v>19:00</v>
+        <v>12:15</v>
       </c>
       <c r="D11" t="str">
-        <v>21:45</v>
+        <v>15:00</v>
       </c>
       <c r="E11" t="str">
         <v/>
       </c>
       <c r="F11" t="str">
-        <v/>
+        <v>IPP (SRN)</v>
       </c>
       <c r="G11" t="str">
-        <v>SAPM-B (VB) / PF (PKB) / ACF (ARS)</v>
+        <v/>
       </c>
       <c r="H11" t="str">
         <v/>
@@ -2957,7 +2957,7 @@
         <v/>
       </c>
       <c r="L11" t="str">
-        <v/>
+        <v>SI-A (AK) / SI-B (PV) / MASA (KKS)</v>
       </c>
     </row>
     <row r="12">
@@ -2968,13 +2968,13 @@
         <v>Sunday</v>
       </c>
       <c r="C12" t="str">
-        <v>09:00</v>
+        <v>15:30</v>
       </c>
       <c r="D12" t="str">
-        <v>11:45</v>
+        <v>18:15</v>
       </c>
       <c r="E12" t="str">
-        <v>SCM-C (RK) / LSS-B (SG)</v>
+        <v/>
       </c>
       <c r="F12" t="str">
         <v/>
@@ -2983,13 +2983,13 @@
         <v/>
       </c>
       <c r="H12" t="str">
-        <v>ACCTP (DS) / DPI (SAA)</v>
+        <v/>
       </c>
       <c r="I12" t="str">
-        <v/>
+        <v>AIB-A (MPS) / CSP (SRA)</v>
       </c>
       <c r="J12" t="str">
-        <v/>
+        <v>PBM-B (SS)</v>
       </c>
       <c r="K12" t="str">
         <v/>
@@ -3000,22 +3000,22 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2024-12-08</v>
+        <v>2024-12-09</v>
       </c>
       <c r="B13" t="str">
-        <v>Sunday</v>
+        <v>Monday</v>
       </c>
       <c r="C13" t="str">
-        <v>12:15</v>
+        <v>15:30</v>
       </c>
       <c r="D13" t="str">
-        <v>15:00</v>
+        <v>18:15</v>
       </c>
       <c r="E13" t="str">
         <v/>
       </c>
       <c r="F13" t="str">
-        <v>IPP (SRN)</v>
+        <v/>
       </c>
       <c r="G13" t="str">
         <v/>
@@ -3027,27 +3027,27 @@
         <v/>
       </c>
       <c r="J13" t="str">
-        <v/>
+        <v>MMT (PN)</v>
       </c>
       <c r="K13" t="str">
         <v/>
       </c>
       <c r="L13" t="str">
-        <v>MTI-A (PV) / MTI-B (AK)</v>
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2024-12-08</v>
+        <v>2024-12-11</v>
       </c>
       <c r="B14" t="str">
-        <v>Sunday</v>
+        <v>Wednesday</v>
       </c>
       <c r="C14" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D14" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E14" t="str">
         <v/>
@@ -3056,16 +3056,16 @@
         <v/>
       </c>
       <c r="G14" t="str">
-        <v/>
+        <v>SAPM-A (ST)</v>
       </c>
       <c r="H14" t="str">
         <v/>
       </c>
       <c r="I14" t="str">
-        <v>AIB-A (MPS) / CSP (SRA)</v>
+        <v/>
       </c>
       <c r="J14" t="str">
-        <v>MBM (JT) / MMT (PN)</v>
+        <v/>
       </c>
       <c r="K14" t="str">
         <v/>
@@ -3076,16 +3076,16 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2024-12-09</v>
+        <v>2024-12-12</v>
       </c>
       <c r="B15" t="str">
-        <v>Monday</v>
+        <v>Thursday</v>
       </c>
       <c r="C15" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D15" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E15" t="str">
         <v/>
@@ -3103,21 +3103,21 @@
         <v/>
       </c>
       <c r="J15" t="str">
-        <v>PBM-A (JJ)</v>
+        <v/>
       </c>
       <c r="K15" t="str">
         <v/>
       </c>
       <c r="L15" t="str">
-        <v/>
+        <v>MASA (KKS)</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2024-12-11</v>
+        <v>2024-12-13</v>
       </c>
       <c r="B16" t="str">
-        <v>Wednesday</v>
+        <v>Friday</v>
       </c>
       <c r="C16" t="str">
         <v>19:00</v>
@@ -3132,10 +3132,10 @@
         <v/>
       </c>
       <c r="G16" t="str">
-        <v>ACF (ARS)</v>
+        <v/>
       </c>
       <c r="H16" t="str">
-        <v/>
+        <v>CCC (DS)</v>
       </c>
       <c r="I16" t="str">
         <v/>
@@ -3152,19 +3152,19 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2024-12-13</v>
+        <v>2024-12-14</v>
       </c>
       <c r="B17" t="str">
-        <v>Friday</v>
+        <v>Saturday</v>
       </c>
       <c r="C17" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D17" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E17" t="str">
-        <v>LSS-A (GN)</v>
+        <v/>
       </c>
       <c r="F17" t="str">
         <v/>
@@ -3182,7 +3182,7 @@
         <v/>
       </c>
       <c r="K17" t="str">
-        <v/>
+        <v>LSO (PNR)</v>
       </c>
       <c r="L17" t="str">
         <v/>
@@ -3208,7 +3208,7 @@
         <v/>
       </c>
       <c r="G18" t="str">
-        <v>ACF (ARS)</v>
+        <v>SAPM-A (ST)</v>
       </c>
       <c r="H18" t="str">
         <v/>
@@ -3234,13 +3234,13 @@
         <v>Sunday</v>
       </c>
       <c r="C19" t="str">
-        <v>09:00</v>
+        <v>12:15</v>
       </c>
       <c r="D19" t="str">
-        <v>11:45</v>
+        <v>15:00</v>
       </c>
       <c r="E19" t="str">
-        <v>LSS-A (GN)</v>
+        <v/>
       </c>
       <c r="F19" t="str">
         <v/>
@@ -3261,7 +3261,7 @@
         <v/>
       </c>
       <c r="L19" t="str">
-        <v/>
+        <v>MASA (KKS)</v>
       </c>
     </row>
     <row r="20">
@@ -3293,7 +3293,7 @@
         <v/>
       </c>
       <c r="J20" t="str">
-        <v>PBM-A (JJ)</v>
+        <v>PBM-A (JJ) / MMT (PN)</v>
       </c>
       <c r="K20" t="str">
         <v/>
@@ -3304,10 +3304,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2024-12-22</v>
+        <v>2024-12-16</v>
       </c>
       <c r="B21" t="str">
-        <v>Sunday</v>
+        <v>Monday</v>
       </c>
       <c r="C21" t="str">
         <v>15:30</v>
@@ -3331,7 +3331,7 @@
         <v/>
       </c>
       <c r="J21" t="str">
-        <v>PBM-A (JJ)</v>
+        <v>SM (PB) / PBM-A (JJ) / PBM-B (SS)</v>
       </c>
       <c r="K21" t="str">
         <v/>
@@ -3342,16 +3342,16 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2024-12-23</v>
+        <v>2024-12-18</v>
       </c>
       <c r="B22" t="str">
-        <v>Monday</v>
+        <v>Wednesday</v>
       </c>
       <c r="C22" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D22" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E22" t="str">
         <v/>
@@ -3360,7 +3360,7 @@
         <v/>
       </c>
       <c r="G22" t="str">
-        <v/>
+        <v>SAPM-B (VB) / ACF (ARS)</v>
       </c>
       <c r="H22" t="str">
         <v/>
@@ -3369,7 +3369,7 @@
         <v/>
       </c>
       <c r="J22" t="str">
-        <v>MBM (JT)</v>
+        <v/>
       </c>
       <c r="K22" t="str">
         <v/>
@@ -3380,16 +3380,16 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2024-12-29</v>
+        <v>2024-12-21</v>
       </c>
       <c r="B23" t="str">
-        <v>Sunday</v>
+        <v>Saturday</v>
       </c>
       <c r="C23" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D23" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E23" t="str">
         <v/>
@@ -3398,7 +3398,7 @@
         <v/>
       </c>
       <c r="G23" t="str">
-        <v/>
+        <v>SAPM-B (VB) / ACF (ARS)</v>
       </c>
       <c r="H23" t="str">
         <v/>
@@ -3407,7 +3407,7 @@
         <v/>
       </c>
       <c r="J23" t="str">
-        <v>MBM (JT)</v>
+        <v/>
       </c>
       <c r="K23" t="str">
         <v/>
@@ -3418,10 +3418,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2024-12-30</v>
+        <v>2024-12-22</v>
       </c>
       <c r="B24" t="str">
-        <v>Monday</v>
+        <v>Sunday</v>
       </c>
       <c r="C24" t="str">
         <v>15:30</v>
@@ -3445,7 +3445,7 @@
         <v/>
       </c>
       <c r="J24" t="str">
-        <v>MBM (JT) / SM (PB)</v>
+        <v>SM (PB) / PBM-B (SS)</v>
       </c>
       <c r="K24" t="str">
         <v/>
@@ -3456,16 +3456,16 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2024-12-31</v>
+        <v>2024-12-23</v>
       </c>
       <c r="B25" t="str">
-        <v>Tuesday</v>
+        <v>Monday</v>
       </c>
       <c r="C25" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D25" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E25" t="str">
         <v/>
@@ -3480,10 +3480,10 @@
         <v/>
       </c>
       <c r="I25" t="str">
-        <v>AIB-A (MPS) / AIB-B (VK)</v>
+        <v/>
       </c>
       <c r="J25" t="str">
-        <v/>
+        <v>MBM (JT)</v>
       </c>
       <c r="K25" t="str">
         <v/>
@@ -3494,10 +3494,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2025-01-01</v>
+        <v>2024-12-24</v>
       </c>
       <c r="B26" t="str">
-        <v>Wednesday</v>
+        <v>Tuesday</v>
       </c>
       <c r="C26" t="str">
         <v>19:00</v>
@@ -3512,19 +3512,19 @@
         <v/>
       </c>
       <c r="G26" t="str">
-        <v>PF (PKB)</v>
+        <v/>
       </c>
       <c r="H26" t="str">
         <v/>
       </c>
       <c r="I26" t="str">
-        <v/>
+        <v>AIB-A (MPS)</v>
       </c>
       <c r="J26" t="str">
         <v/>
       </c>
       <c r="K26" t="str">
-        <v>LSO (PNR)</v>
+        <v/>
       </c>
       <c r="L26" t="str">
         <v/>
@@ -3532,10 +3532,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2025-01-02</v>
+        <v>2024-12-25</v>
       </c>
       <c r="B27" t="str">
-        <v>Thursday</v>
+        <v>Wednesday</v>
       </c>
       <c r="C27" t="str">
         <v>19:00</v>
@@ -3547,10 +3547,10 @@
         <v/>
       </c>
       <c r="F27" t="str">
-        <v>GT (AG) / ABMBM (VPV)</v>
+        <v/>
       </c>
       <c r="G27" t="str">
-        <v/>
+        <v>PF (PKB)</v>
       </c>
       <c r="H27" t="str">
         <v/>
@@ -3570,7 +3570,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2025-01-03</v>
+        <v>2024-12-27</v>
       </c>
       <c r="B28" t="str">
         <v>Friday</v>
@@ -3582,7 +3582,7 @@
         <v>21:45</v>
       </c>
       <c r="E28" t="str">
-        <v>LSS-A (GN)</v>
+        <v>SCM-B (SSP) / SCM-C (RK)</v>
       </c>
       <c r="F28" t="str">
         <v/>
@@ -3591,7 +3591,7 @@
         <v/>
       </c>
       <c r="H28" t="str">
-        <v>ACCTP (DS)</v>
+        <v/>
       </c>
       <c r="I28" t="str">
         <v/>
@@ -3608,16 +3608,16 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2025-01-04</v>
+        <v>2024-12-28</v>
       </c>
       <c r="B29" t="str">
         <v>Saturday</v>
       </c>
       <c r="C29" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D29" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E29" t="str">
         <v/>
@@ -3626,7 +3626,7 @@
         <v/>
       </c>
       <c r="G29" t="str">
-        <v/>
+        <v>PF (PKB)</v>
       </c>
       <c r="H29" t="str">
         <v/>
@@ -3638,7 +3638,7 @@
         <v/>
       </c>
       <c r="K29" t="str">
-        <v>LSO (PNR)</v>
+        <v/>
       </c>
       <c r="L29" t="str">
         <v/>
@@ -3646,25 +3646,25 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2025-01-04</v>
+        <v>2024-12-29</v>
       </c>
       <c r="B30" t="str">
-        <v>Saturday</v>
+        <v>Sunday</v>
       </c>
       <c r="C30" t="str">
-        <v>19:00</v>
+        <v>09:00</v>
       </c>
       <c r="D30" t="str">
-        <v>21:45</v>
+        <v>11:45</v>
       </c>
       <c r="E30" t="str">
-        <v/>
+        <v>SCM-B (SSP) / SCM-C (RK)</v>
       </c>
       <c r="F30" t="str">
         <v/>
       </c>
       <c r="G30" t="str">
-        <v>PF (PKB)</v>
+        <v/>
       </c>
       <c r="H30" t="str">
         <v/>
@@ -3684,19 +3684,19 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2025-01-05</v>
+        <v>2024-12-29</v>
       </c>
       <c r="B31" t="str">
         <v>Sunday</v>
       </c>
       <c r="C31" t="str">
-        <v>09:00</v>
+        <v>15:30</v>
       </c>
       <c r="D31" t="str">
-        <v>11:45</v>
+        <v>18:15</v>
       </c>
       <c r="E31" t="str">
-        <v>LSS-A (GN)</v>
+        <v/>
       </c>
       <c r="F31" t="str">
         <v/>
@@ -3705,13 +3705,13 @@
         <v/>
       </c>
       <c r="H31" t="str">
-        <v>ACCTP (DS)</v>
+        <v/>
       </c>
       <c r="I31" t="str">
-        <v/>
+        <v>AIB-A (MPS)</v>
       </c>
       <c r="J31" t="str">
-        <v/>
+        <v>MBM (JT)</v>
       </c>
       <c r="K31" t="str">
         <v/>
@@ -3722,22 +3722,22 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2025-01-05</v>
+        <v>2024-12-30</v>
       </c>
       <c r="B32" t="str">
-        <v>Sunday</v>
+        <v>Monday</v>
       </c>
       <c r="C32" t="str">
-        <v>12:15</v>
+        <v>15:30</v>
       </c>
       <c r="D32" t="str">
-        <v>15:00</v>
+        <v>18:15</v>
       </c>
       <c r="E32" t="str">
         <v/>
       </c>
       <c r="F32" t="str">
-        <v>GT (AG) / ABMBM (VPV)</v>
+        <v/>
       </c>
       <c r="G32" t="str">
         <v/>
@@ -3749,7 +3749,7 @@
         <v/>
       </c>
       <c r="J32" t="str">
-        <v/>
+        <v>UOSWTPB (PS)</v>
       </c>
       <c r="K32" t="str">
         <v/>
@@ -3760,16 +3760,16 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2025-01-05</v>
+        <v>2025-01-01</v>
       </c>
       <c r="B33" t="str">
-        <v>Sunday</v>
+        <v>Wednesday</v>
       </c>
       <c r="C33" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D33" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E33" t="str">
         <v/>
@@ -3778,16 +3778,16 @@
         <v/>
       </c>
       <c r="G33" t="str">
-        <v/>
+        <v>ACF (ARS)</v>
       </c>
       <c r="H33" t="str">
         <v/>
       </c>
       <c r="I33" t="str">
-        <v>AIB-A (MPS) / AIB-B (VK)</v>
+        <v/>
       </c>
       <c r="J33" t="str">
-        <v>MBM (JT) / SM (PB)</v>
+        <v/>
       </c>
       <c r="K33" t="str">
         <v/>
@@ -3798,22 +3798,22 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2025-01-06</v>
+        <v>2025-01-02</v>
       </c>
       <c r="B34" t="str">
-        <v>Monday</v>
+        <v>Thursday</v>
       </c>
       <c r="C34" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D34" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E34" t="str">
         <v/>
       </c>
       <c r="F34" t="str">
-        <v/>
+        <v>GT (AG)</v>
       </c>
       <c r="G34" t="str">
         <v/>
@@ -3825,7 +3825,7 @@
         <v/>
       </c>
       <c r="J34" t="str">
-        <v>PBM-B (SS) / MMT (PN)</v>
+        <v/>
       </c>
       <c r="K34" t="str">
         <v/>
@@ -3836,10 +3836,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2025-01-07</v>
+        <v>2025-01-03</v>
       </c>
       <c r="B35" t="str">
-        <v>Tuesday</v>
+        <v>Friday</v>
       </c>
       <c r="C35" t="str">
         <v>19:00</v>
@@ -3848,7 +3848,7 @@
         <v>21:45</v>
       </c>
       <c r="E35" t="str">
-        <v/>
+        <v>SCM-B (SSP) / LSS-A (GN)</v>
       </c>
       <c r="F35" t="str">
         <v/>
@@ -3857,10 +3857,10 @@
         <v/>
       </c>
       <c r="H35" t="str">
-        <v/>
+        <v>CCC (DS)</v>
       </c>
       <c r="I35" t="str">
-        <v>AIB-B (VK)</v>
+        <v/>
       </c>
       <c r="J35" t="str">
         <v/>
@@ -3874,10 +3874,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2025-01-08</v>
+        <v>2025-01-04</v>
       </c>
       <c r="B36" t="str">
-        <v>Wednesday</v>
+        <v>Saturday</v>
       </c>
       <c r="C36" t="str">
         <v>19:00</v>
@@ -3892,7 +3892,7 @@
         <v/>
       </c>
       <c r="G36" t="str">
-        <v>SAPM-A (ST) / SAPM-B (VB) / ACF (ARS)</v>
+        <v>ACF (ARS)</v>
       </c>
       <c r="H36" t="str">
         <v/>
@@ -3912,28 +3912,28 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>2025-01-09</v>
+        <v>2025-01-05</v>
       </c>
       <c r="B37" t="str">
-        <v>Thursday</v>
+        <v>Sunday</v>
       </c>
       <c r="C37" t="str">
-        <v>19:00</v>
+        <v>09:00</v>
       </c>
       <c r="D37" t="str">
-        <v>21:45</v>
+        <v>11:45</v>
       </c>
       <c r="E37" t="str">
-        <v/>
+        <v>SCM-B (SSP) / LSS-A (GN)</v>
       </c>
       <c r="F37" t="str">
-        <v>GT (AG) / IPP (SRN)</v>
+        <v/>
       </c>
       <c r="G37" t="str">
         <v/>
       </c>
       <c r="H37" t="str">
-        <v/>
+        <v>CCC (DS)</v>
       </c>
       <c r="I37" t="str">
         <v/>
@@ -3945,33 +3945,33 @@
         <v/>
       </c>
       <c r="L37" t="str">
-        <v>MTI-A (PV) / MASA (KKS)</v>
+        <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>2025-01-10</v>
+        <v>2025-01-05</v>
       </c>
       <c r="B38" t="str">
-        <v>Friday</v>
+        <v>Sunday</v>
       </c>
       <c r="C38" t="str">
-        <v>19:00</v>
+        <v>12:15</v>
       </c>
       <c r="D38" t="str">
-        <v>21:45</v>
+        <v>15:00</v>
       </c>
       <c r="E38" t="str">
-        <v>SCM-B (SSP)</v>
+        <v/>
       </c>
       <c r="F38" t="str">
-        <v/>
+        <v>GT (AG)</v>
       </c>
       <c r="G38" t="str">
         <v/>
       </c>
       <c r="H38" t="str">
-        <v>CCC (DS)</v>
+        <v/>
       </c>
       <c r="I38" t="str">
         <v/>
@@ -3983,21 +3983,21 @@
         <v/>
       </c>
       <c r="L38" t="str">
-        <v/>
+        <v>SI-A (AK)</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>2025-01-11</v>
+        <v>2025-01-05</v>
       </c>
       <c r="B39" t="str">
-        <v>Saturday</v>
+        <v>Sunday</v>
       </c>
       <c r="C39" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D39" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E39" t="str">
         <v/>
@@ -4006,7 +4006,7 @@
         <v/>
       </c>
       <c r="G39" t="str">
-        <v>SAPM-A (ST) / SAPM-B (VB) / ACF (ARS)</v>
+        <v/>
       </c>
       <c r="H39" t="str">
         <v/>
@@ -4015,7 +4015,7 @@
         <v/>
       </c>
       <c r="J39" t="str">
-        <v/>
+        <v>UOSWTPB (PS)</v>
       </c>
       <c r="K39" t="str">
         <v/>
@@ -4026,19 +4026,19 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>2025-01-12</v>
+        <v>2025-01-06</v>
       </c>
       <c r="B40" t="str">
-        <v>Sunday</v>
+        <v>Monday</v>
       </c>
       <c r="C40" t="str">
-        <v>09:00</v>
+        <v>15:30</v>
       </c>
       <c r="D40" t="str">
-        <v>11:45</v>
+        <v>18:15</v>
       </c>
       <c r="E40" t="str">
-        <v>SCM-A (ASS) / SCM-B (SSP) / LSS-A (GN)</v>
+        <v/>
       </c>
       <c r="F40" t="str">
         <v/>
@@ -4047,13 +4047,13 @@
         <v/>
       </c>
       <c r="H40" t="str">
-        <v>CCC (DS)</v>
+        <v/>
       </c>
       <c r="I40" t="str">
         <v/>
       </c>
       <c r="J40" t="str">
-        <v/>
+        <v>MBM (JT) / PBM-A (JJ) / MMT (PN)</v>
       </c>
       <c r="K40" t="str">
         <v/>
@@ -4064,22 +4064,22 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>2025-01-12</v>
+        <v>2025-01-07</v>
       </c>
       <c r="B41" t="str">
-        <v>Sunday</v>
+        <v>Tuesday</v>
       </c>
       <c r="C41" t="str">
-        <v>12:15</v>
+        <v>19:00</v>
       </c>
       <c r="D41" t="str">
-        <v>15:00</v>
+        <v>21:45</v>
       </c>
       <c r="E41" t="str">
         <v/>
       </c>
       <c r="F41" t="str">
-        <v>GT (AG) / IPP (SRN)</v>
+        <v/>
       </c>
       <c r="G41" t="str">
         <v/>
@@ -4088,7 +4088,7 @@
         <v/>
       </c>
       <c r="I41" t="str">
-        <v/>
+        <v>AIB-B (VK)</v>
       </c>
       <c r="J41" t="str">
         <v/>
@@ -4097,21 +4097,21 @@
         <v/>
       </c>
       <c r="L41" t="str">
-        <v>MTI-A (PV) / MASA (KKS)</v>
+        <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>2025-01-12</v>
+        <v>2025-01-08</v>
       </c>
       <c r="B42" t="str">
-        <v>Sunday</v>
+        <v>Wednesday</v>
       </c>
       <c r="C42" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D42" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E42" t="str">
         <v/>
@@ -4120,19 +4120,19 @@
         <v/>
       </c>
       <c r="G42" t="str">
-        <v/>
+        <v>SAPM-A (ST) / ACF (ARS)</v>
       </c>
       <c r="H42" t="str">
         <v/>
       </c>
       <c r="I42" t="str">
-        <v>AIB-B (VK)</v>
+        <v/>
       </c>
       <c r="J42" t="str">
-        <v>PBM-B (SS) / MMT (PN)</v>
+        <v/>
       </c>
       <c r="K42" t="str">
-        <v/>
+        <v>LSO (PNR)</v>
       </c>
       <c r="L42" t="str">
         <v/>
@@ -4140,22 +4140,22 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>2025-01-13</v>
+        <v>2025-01-09</v>
       </c>
       <c r="B43" t="str">
-        <v>Monday</v>
+        <v>Thursday</v>
       </c>
       <c r="C43" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D43" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E43" t="str">
         <v/>
       </c>
       <c r="F43" t="str">
-        <v/>
+        <v>IPP (SRN)</v>
       </c>
       <c r="G43" t="str">
         <v/>
@@ -4167,21 +4167,21 @@
         <v/>
       </c>
       <c r="J43" t="str">
-        <v>PBM-A (JJ) / PBM-B (SS) / MMT (PN)</v>
+        <v/>
       </c>
       <c r="K43" t="str">
         <v/>
       </c>
       <c r="L43" t="str">
-        <v/>
+        <v>MTI-B (AK) / MASA (KKS)</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>2025-01-14</v>
+        <v>2025-01-10</v>
       </c>
       <c r="B44" t="str">
-        <v>Tuesday</v>
+        <v>Friday</v>
       </c>
       <c r="C44" t="str">
         <v>19:00</v>
@@ -4190,7 +4190,7 @@
         <v>21:45</v>
       </c>
       <c r="E44" t="str">
-        <v/>
+        <v>LSS-A (GN) / LSS-B (SG)</v>
       </c>
       <c r="F44" t="str">
         <v/>
@@ -4199,10 +4199,10 @@
         <v/>
       </c>
       <c r="H44" t="str">
-        <v/>
+        <v>CCC (DS)</v>
       </c>
       <c r="I44" t="str">
-        <v>CSP (SRA)</v>
+        <v/>
       </c>
       <c r="J44" t="str">
         <v/>
@@ -4216,16 +4216,16 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>2025-01-15</v>
+        <v>2025-01-11</v>
       </c>
       <c r="B45" t="str">
-        <v>Wednesday</v>
+        <v>Saturday</v>
       </c>
       <c r="C45" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D45" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -4234,7 +4234,7 @@
         <v/>
       </c>
       <c r="G45" t="str">
-        <v>SAPM-B (VB) / PF (PKB) / ACF (ARS)</v>
+        <v/>
       </c>
       <c r="H45" t="str">
         <v/>
@@ -4246,7 +4246,7 @@
         <v/>
       </c>
       <c r="K45" t="str">
-        <v/>
+        <v>LSO (PNR)</v>
       </c>
       <c r="L45" t="str">
         <v/>
@@ -4254,10 +4254,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>2025-01-16</v>
+        <v>2025-01-11</v>
       </c>
       <c r="B46" t="str">
-        <v>Thursday</v>
+        <v>Saturday</v>
       </c>
       <c r="C46" t="str">
         <v>19:00</v>
@@ -4269,10 +4269,10 @@
         <v/>
       </c>
       <c r="F46" t="str">
-        <v>GT (AG) / IPP (SRN)</v>
+        <v/>
       </c>
       <c r="G46" t="str">
-        <v/>
+        <v>SAPM-A (ST) / ACF (ARS)</v>
       </c>
       <c r="H46" t="str">
         <v/>
@@ -4287,24 +4287,24 @@
         <v/>
       </c>
       <c r="L46" t="str">
-        <v>SI-A (AK) / MASA (KKS)</v>
+        <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>2025-01-17</v>
+        <v>2025-01-12</v>
       </c>
       <c r="B47" t="str">
-        <v>Friday</v>
+        <v>Sunday</v>
       </c>
       <c r="C47" t="str">
-        <v>19:00</v>
+        <v>09:00</v>
       </c>
       <c r="D47" t="str">
-        <v>21:45</v>
+        <v>11:45</v>
       </c>
       <c r="E47" t="str">
-        <v>SCM-B (SSP) / SCM-C (RK)</v>
+        <v>LSS-A (GN) / LSS-B (SG)</v>
       </c>
       <c r="F47" t="str">
         <v/>
@@ -4313,7 +4313,7 @@
         <v/>
       </c>
       <c r="H47" t="str">
-        <v>ACCTP (DS) / DPI (SAA)</v>
+        <v>CCC (DS)</v>
       </c>
       <c r="I47" t="str">
         <v/>
@@ -4330,25 +4330,25 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>2025-01-18</v>
+        <v>2025-01-12</v>
       </c>
       <c r="B48" t="str">
-        <v>Saturday</v>
+        <v>Sunday</v>
       </c>
       <c r="C48" t="str">
-        <v>19:00</v>
+        <v>12:15</v>
       </c>
       <c r="D48" t="str">
-        <v>21:45</v>
+        <v>15:00</v>
       </c>
       <c r="E48" t="str">
         <v/>
       </c>
       <c r="F48" t="str">
-        <v/>
+        <v>IPP (SRN)</v>
       </c>
       <c r="G48" t="str">
-        <v>SAPM-B (VB) / PF (PKB) / ACF (ARS)</v>
+        <v/>
       </c>
       <c r="H48" t="str">
         <v/>
@@ -4363,24 +4363,24 @@
         <v/>
       </c>
       <c r="L48" t="str">
-        <v/>
+        <v>MTI-B (AK) / MASA (KKS)</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>2025-01-19</v>
+        <v>2025-01-12</v>
       </c>
       <c r="B49" t="str">
         <v>Sunday</v>
       </c>
       <c r="C49" t="str">
-        <v>09:00</v>
+        <v>15:30</v>
       </c>
       <c r="D49" t="str">
-        <v>11:45</v>
+        <v>18:15</v>
       </c>
       <c r="E49" t="str">
-        <v>SCM-B (SSP) / SCM-C (RK)</v>
+        <v/>
       </c>
       <c r="F49" t="str">
         <v/>
@@ -4389,13 +4389,13 @@
         <v/>
       </c>
       <c r="H49" t="str">
-        <v>ACCTP (DS) / DPI (SAA)</v>
+        <v/>
       </c>
       <c r="I49" t="str">
-        <v/>
+        <v>AIB-B (VK)</v>
       </c>
       <c r="J49" t="str">
-        <v/>
+        <v>MBM (JT) / PBM-A (JJ) / MMT (PN)</v>
       </c>
       <c r="K49" t="str">
         <v/>
@@ -4406,22 +4406,22 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>2025-01-19</v>
+        <v>2025-01-13</v>
       </c>
       <c r="B50" t="str">
-        <v>Sunday</v>
+        <v>Monday</v>
       </c>
       <c r="C50" t="str">
-        <v>12:15</v>
+        <v>15:30</v>
       </c>
       <c r="D50" t="str">
-        <v>15:00</v>
+        <v>18:15</v>
       </c>
       <c r="E50" t="str">
         <v/>
       </c>
       <c r="F50" t="str">
-        <v>GT (AG) / IPP (SRN)</v>
+        <v/>
       </c>
       <c r="G50" t="str">
         <v/>
@@ -4433,27 +4433,27 @@
         <v/>
       </c>
       <c r="J50" t="str">
-        <v/>
+        <v>SM (PB) / UOSWTPB (PS)</v>
       </c>
       <c r="K50" t="str">
         <v/>
       </c>
       <c r="L50" t="str">
-        <v>SI-A (AK) / MASA (KKS)</v>
+        <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>2025-01-19</v>
+        <v>2025-01-14</v>
       </c>
       <c r="B51" t="str">
-        <v>Sunday</v>
+        <v>Tuesday</v>
       </c>
       <c r="C51" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D51" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E51" t="str">
         <v/>
@@ -4471,7 +4471,7 @@
         <v>CSP (SRA)</v>
       </c>
       <c r="J51" t="str">
-        <v>PBM-A (JJ) / PBM-B (SS) / MMT (PN)</v>
+        <v/>
       </c>
       <c r="K51" t="str">
         <v/>
@@ -4482,16 +4482,16 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>2025-01-20</v>
+        <v>2025-01-15</v>
       </c>
       <c r="B52" t="str">
-        <v>Monday</v>
+        <v>Wednesday</v>
       </c>
       <c r="C52" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D52" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E52" t="str">
         <v/>
@@ -4500,7 +4500,7 @@
         <v/>
       </c>
       <c r="G52" t="str">
-        <v/>
+        <v>AMA (PKB) / SAPM-A (ST) / SAPM-B (VB)</v>
       </c>
       <c r="H52" t="str">
         <v/>
@@ -4509,7 +4509,7 @@
         <v/>
       </c>
       <c r="J52" t="str">
-        <v>MBM (JT) / UOSWTPB (PS)</v>
+        <v/>
       </c>
       <c r="K52" t="str">
         <v/>
@@ -4520,10 +4520,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>2025-01-21</v>
+        <v>2025-01-16</v>
       </c>
       <c r="B53" t="str">
-        <v>Tuesday</v>
+        <v>Thursday</v>
       </c>
       <c r="C53" t="str">
         <v>19:00</v>
@@ -4535,7 +4535,7 @@
         <v/>
       </c>
       <c r="F53" t="str">
-        <v/>
+        <v>GT (AG) / IPP (SRN) / ABMBM (VPV)</v>
       </c>
       <c r="G53" t="str">
         <v/>
@@ -4544,7 +4544,7 @@
         <v/>
       </c>
       <c r="I53" t="str">
-        <v>CSP (SRA)</v>
+        <v/>
       </c>
       <c r="J53" t="str">
         <v/>
@@ -4553,15 +4553,15 @@
         <v/>
       </c>
       <c r="L53" t="str">
-        <v/>
+        <v>MASA (KKS)</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>2025-01-22</v>
+        <v>2025-01-17</v>
       </c>
       <c r="B54" t="str">
-        <v>Wednesday</v>
+        <v>Friday</v>
       </c>
       <c r="C54" t="str">
         <v>19:00</v>
@@ -4570,16 +4570,16 @@
         <v>21:45</v>
       </c>
       <c r="E54" t="str">
-        <v/>
+        <v>SCM-B (SSP)</v>
       </c>
       <c r="F54" t="str">
         <v/>
       </c>
       <c r="G54" t="str">
-        <v>AMA (PKB) / SAPM-A (ST)</v>
+        <v/>
       </c>
       <c r="H54" t="str">
-        <v/>
+        <v>DPI (SAA)</v>
       </c>
       <c r="I54" t="str">
         <v/>
@@ -4596,10 +4596,10 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>2025-01-24</v>
+        <v>2025-01-18</v>
       </c>
       <c r="B55" t="str">
-        <v>Friday</v>
+        <v>Saturday</v>
       </c>
       <c r="C55" t="str">
         <v>19:00</v>
@@ -4608,16 +4608,16 @@
         <v>21:45</v>
       </c>
       <c r="E55" t="str">
-        <v>SCM-A (ASS) / LSS-A (GN) / LSS-B (SG)</v>
+        <v/>
       </c>
       <c r="F55" t="str">
         <v/>
       </c>
       <c r="G55" t="str">
-        <v/>
+        <v>AMA (PKB) / SAPM-A (ST) / SAPM-B (VB)</v>
       </c>
       <c r="H55" t="str">
-        <v>CCC (DS)</v>
+        <v/>
       </c>
       <c r="I55" t="str">
         <v/>
@@ -4634,19 +4634,19 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>2025-01-25</v>
+        <v>2025-01-19</v>
       </c>
       <c r="B56" t="str">
-        <v>Saturday</v>
+        <v>Sunday</v>
       </c>
       <c r="C56" t="str">
-        <v>15:30</v>
+        <v>09:00</v>
       </c>
       <c r="D56" t="str">
-        <v>18:15</v>
+        <v>11:45</v>
       </c>
       <c r="E56" t="str">
-        <v/>
+        <v>SCM-B (SSP)</v>
       </c>
       <c r="F56" t="str">
         <v/>
@@ -4655,7 +4655,7 @@
         <v/>
       </c>
       <c r="H56" t="str">
-        <v/>
+        <v>DPI (SAA)</v>
       </c>
       <c r="I56" t="str">
         <v/>
@@ -4664,7 +4664,7 @@
         <v/>
       </c>
       <c r="K56" t="str">
-        <v>LSO (PNR)</v>
+        <v/>
       </c>
       <c r="L56" t="str">
         <v/>
@@ -4672,25 +4672,25 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>2025-01-25</v>
+        <v>2025-01-19</v>
       </c>
       <c r="B57" t="str">
-        <v>Saturday</v>
+        <v>Sunday</v>
       </c>
       <c r="C57" t="str">
-        <v>19:00</v>
+        <v>12:15</v>
       </c>
       <c r="D57" t="str">
-        <v>21:45</v>
+        <v>15:00</v>
       </c>
       <c r="E57" t="str">
         <v/>
       </c>
       <c r="F57" t="str">
-        <v/>
+        <v>GT (AG) / IPP (SRN) / ABMBM (VPV)</v>
       </c>
       <c r="G57" t="str">
-        <v>AMA (PKB) / SAPM-A (ST)</v>
+        <v/>
       </c>
       <c r="H57" t="str">
         <v/>
@@ -4705,24 +4705,24 @@
         <v/>
       </c>
       <c r="L57" t="str">
-        <v/>
+        <v>MASA (KKS)</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>2025-01-26</v>
+        <v>2025-01-19</v>
       </c>
       <c r="B58" t="str">
         <v>Sunday</v>
       </c>
       <c r="C58" t="str">
-        <v>09:00</v>
+        <v>15:30</v>
       </c>
       <c r="D58" t="str">
-        <v>11:45</v>
+        <v>18:15</v>
       </c>
       <c r="E58" t="str">
-        <v>SCM-A (ASS) / LSS-A (GN) / LSS-B (SG)</v>
+        <v/>
       </c>
       <c r="F58" t="str">
         <v/>
@@ -4731,13 +4731,13 @@
         <v/>
       </c>
       <c r="H58" t="str">
-        <v>CCC (DS)</v>
+        <v/>
       </c>
       <c r="I58" t="str">
-        <v/>
+        <v>CSP (SRA)</v>
       </c>
       <c r="J58" t="str">
-        <v/>
+        <v>SM (PB) / UOSWTPB (PS)</v>
       </c>
       <c r="K58" t="str">
         <v/>
@@ -4748,10 +4748,10 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>2025-01-26</v>
+        <v>2025-01-20</v>
       </c>
       <c r="B59" t="str">
-        <v>Sunday</v>
+        <v>Monday</v>
       </c>
       <c r="C59" t="str">
         <v>15:30</v>
@@ -4772,10 +4772,10 @@
         <v/>
       </c>
       <c r="I59" t="str">
-        <v>CSP (SRA)</v>
+        <v/>
       </c>
       <c r="J59" t="str">
-        <v>MBM (JT) / UOSWTPB (PS)</v>
+        <v>MBM (JT) / MMT (PN)</v>
       </c>
       <c r="K59" t="str">
         <v/>
@@ -4786,16 +4786,16 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>2025-01-27</v>
+        <v>2025-01-21</v>
       </c>
       <c r="B60" t="str">
-        <v>Monday</v>
+        <v>Tuesday</v>
       </c>
       <c r="C60" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D60" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E60" t="str">
         <v/>
@@ -4810,10 +4810,10 @@
         <v/>
       </c>
       <c r="I60" t="str">
-        <v/>
+        <v>AIB-B (VK)</v>
       </c>
       <c r="J60" t="str">
-        <v>MBM (JT) / PBM-A (JJ)</v>
+        <v/>
       </c>
       <c r="K60" t="str">
         <v/>
@@ -4824,10 +4824,10 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>2025-01-28</v>
+        <v>2025-01-22</v>
       </c>
       <c r="B61" t="str">
-        <v>Tuesday</v>
+        <v>Wednesday</v>
       </c>
       <c r="C61" t="str">
         <v>19:00</v>
@@ -4842,13 +4842,13 @@
         <v/>
       </c>
       <c r="G61" t="str">
-        <v/>
+        <v>PF (PKB) / ACF (ARS)</v>
       </c>
       <c r="H61" t="str">
         <v/>
       </c>
       <c r="I61" t="str">
-        <v>AIB-B (VK)</v>
+        <v/>
       </c>
       <c r="J61" t="str">
         <v/>
@@ -4862,10 +4862,10 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>2025-01-29</v>
+        <v>2025-01-23</v>
       </c>
       <c r="B62" t="str">
-        <v>Wednesday</v>
+        <v>Thursday</v>
       </c>
       <c r="C62" t="str">
         <v>19:00</v>
@@ -4877,10 +4877,10 @@
         <v/>
       </c>
       <c r="F62" t="str">
-        <v/>
+        <v>ABMBM (VPV)</v>
       </c>
       <c r="G62" t="str">
-        <v>AMA (PKB)</v>
+        <v/>
       </c>
       <c r="H62" t="str">
         <v/>
@@ -4900,10 +4900,10 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>2025-01-30</v>
+        <v>2025-01-24</v>
       </c>
       <c r="B63" t="str">
-        <v>Thursday</v>
+        <v>Friday</v>
       </c>
       <c r="C63" t="str">
         <v>19:00</v>
@@ -4912,7 +4912,7 @@
         <v>21:45</v>
       </c>
       <c r="E63" t="str">
-        <v/>
+        <v>LSS-A (GN) / LSS-B (SG)</v>
       </c>
       <c r="F63" t="str">
         <v/>
@@ -4921,7 +4921,7 @@
         <v/>
       </c>
       <c r="H63" t="str">
-        <v/>
+        <v>ACCTP (DS) / DPI (SAA)</v>
       </c>
       <c r="I63" t="str">
         <v/>
@@ -4933,15 +4933,15 @@
         <v/>
       </c>
       <c r="L63" t="str">
-        <v>SI-B (PV)</v>
+        <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>2025-01-31</v>
+        <v>2025-01-25</v>
       </c>
       <c r="B64" t="str">
-        <v>Friday</v>
+        <v>Saturday</v>
       </c>
       <c r="C64" t="str">
         <v>19:00</v>
@@ -4950,13 +4950,13 @@
         <v>21:45</v>
       </c>
       <c r="E64" t="str">
-        <v>SCM-A (ASS) / LSS-A (GN) / LSS-B (SG)</v>
+        <v/>
       </c>
       <c r="F64" t="str">
         <v/>
       </c>
       <c r="G64" t="str">
-        <v/>
+        <v>PF (PKB) / ACF (ARS)</v>
       </c>
       <c r="H64" t="str">
         <v/>
@@ -4976,28 +4976,28 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>2025-02-01</v>
+        <v>2025-01-26</v>
       </c>
       <c r="B65" t="str">
-        <v>Saturday</v>
+        <v>Sunday</v>
       </c>
       <c r="C65" t="str">
-        <v>19:00</v>
+        <v>09:00</v>
       </c>
       <c r="D65" t="str">
-        <v>21:45</v>
+        <v>11:45</v>
       </c>
       <c r="E65" t="str">
-        <v/>
+        <v>LSS-A (GN) / LSS-B (SG)</v>
       </c>
       <c r="F65" t="str">
         <v/>
       </c>
       <c r="G65" t="str">
-        <v>AMA (PKB)</v>
+        <v/>
       </c>
       <c r="H65" t="str">
-        <v/>
+        <v>ACCTP (DS) / DPI (SAA)</v>
       </c>
       <c r="I65" t="str">
         <v/>
@@ -5014,22 +5014,22 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>2025-02-02</v>
+        <v>2025-01-26</v>
       </c>
       <c r="B66" t="str">
         <v>Sunday</v>
       </c>
       <c r="C66" t="str">
-        <v>09:00</v>
+        <v>12:15</v>
       </c>
       <c r="D66" t="str">
-        <v>11:45</v>
+        <v>15:00</v>
       </c>
       <c r="E66" t="str">
-        <v>SCM-A (ASS) / LSS-A (GN) / LSS-B (SG)</v>
+        <v/>
       </c>
       <c r="F66" t="str">
-        <v/>
+        <v>ABMBM (VPV)</v>
       </c>
       <c r="G66" t="str">
         <v/>
@@ -5052,16 +5052,16 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>2025-02-02</v>
+        <v>2025-01-26</v>
       </c>
       <c r="B67" t="str">
         <v>Sunday</v>
       </c>
       <c r="C67" t="str">
-        <v>12:15</v>
+        <v>15:30</v>
       </c>
       <c r="D67" t="str">
-        <v>15:00</v>
+        <v>18:15</v>
       </c>
       <c r="E67" t="str">
         <v/>
@@ -5076,24 +5076,24 @@
         <v/>
       </c>
       <c r="I67" t="str">
-        <v/>
+        <v>AIB-B (VK)</v>
       </c>
       <c r="J67" t="str">
-        <v/>
+        <v>MBM (JT) / MMT (PN) / UOSWTPB (PS)</v>
       </c>
       <c r="K67" t="str">
         <v/>
       </c>
       <c r="L67" t="str">
-        <v>SI-B (PV)</v>
+        <v/>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>2025-02-02</v>
+        <v>2025-01-27</v>
       </c>
       <c r="B68" t="str">
-        <v>Sunday</v>
+        <v>Monday</v>
       </c>
       <c r="C68" t="str">
         <v>15:30</v>
@@ -5114,7 +5114,7 @@
         <v/>
       </c>
       <c r="I68" t="str">
-        <v>AIB-B (VK)</v>
+        <v/>
       </c>
       <c r="J68" t="str">
         <v>MBM (JT) / PBM-A (JJ)</v>
@@ -5128,16 +5128,16 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>2025-02-03</v>
+        <v>2025-01-29</v>
       </c>
       <c r="B69" t="str">
-        <v>Monday</v>
+        <v>Wednesday</v>
       </c>
       <c r="C69" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D69" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E69" t="str">
         <v/>
@@ -5146,7 +5146,7 @@
         <v/>
       </c>
       <c r="G69" t="str">
-        <v/>
+        <v>AMA (PKB)</v>
       </c>
       <c r="H69" t="str">
         <v/>
@@ -5155,10 +5155,10 @@
         <v/>
       </c>
       <c r="J69" t="str">
-        <v>MBM (JT) / MMT (PN) / UOSWTPB (PS)</v>
+        <v/>
       </c>
       <c r="K69" t="str">
-        <v/>
+        <v>LSO (PNR)</v>
       </c>
       <c r="L69" t="str">
         <v/>
@@ -5166,10 +5166,10 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>2025-02-05</v>
+        <v>2025-01-30</v>
       </c>
       <c r="B70" t="str">
-        <v>Wednesday</v>
+        <v>Thursday</v>
       </c>
       <c r="C70" t="str">
         <v>19:00</v>
@@ -5181,10 +5181,10 @@
         <v/>
       </c>
       <c r="F70" t="str">
-        <v/>
+        <v>GT (AG)</v>
       </c>
       <c r="G70" t="str">
-        <v>AMA (PKB)</v>
+        <v/>
       </c>
       <c r="H70" t="str">
         <v/>
@@ -5199,15 +5199,15 @@
         <v/>
       </c>
       <c r="L70" t="str">
-        <v/>
+        <v>SI-A (AK)</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>2025-02-06</v>
+        <v>2025-01-31</v>
       </c>
       <c r="B71" t="str">
-        <v>Thursday</v>
+        <v>Friday</v>
       </c>
       <c r="C71" t="str">
         <v>19:00</v>
@@ -5216,16 +5216,16 @@
         <v>21:45</v>
       </c>
       <c r="E71" t="str">
-        <v/>
+        <v>SCM-C (RK) / LSS-B (SG)</v>
       </c>
       <c r="F71" t="str">
-        <v>GT (AG) / IPP (SRN)</v>
+        <v/>
       </c>
       <c r="G71" t="str">
         <v/>
       </c>
       <c r="H71" t="str">
-        <v/>
+        <v>CCC (DS)</v>
       </c>
       <c r="I71" t="str">
         <v/>
@@ -5242,19 +5242,19 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>2025-02-07</v>
+        <v>2025-02-01</v>
       </c>
       <c r="B72" t="str">
-        <v>Friday</v>
+        <v>Saturday</v>
       </c>
       <c r="C72" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D72" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E72" t="str">
-        <v>SCM-A (ASS) / LSS-A (GN) / LSS-B (SG)</v>
+        <v/>
       </c>
       <c r="F72" t="str">
         <v/>
@@ -5272,7 +5272,7 @@
         <v/>
       </c>
       <c r="K72" t="str">
-        <v/>
+        <v>LSO (PNR)</v>
       </c>
       <c r="L72" t="str">
         <v/>
@@ -5280,7 +5280,7 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>2025-02-08</v>
+        <v>2025-02-01</v>
       </c>
       <c r="B73" t="str">
         <v>Saturday</v>
@@ -5318,7 +5318,7 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>2025-02-09</v>
+        <v>2025-02-02</v>
       </c>
       <c r="B74" t="str">
         <v>Sunday</v>
@@ -5330,7 +5330,7 @@
         <v>11:45</v>
       </c>
       <c r="E74" t="str">
-        <v>SCM-A (ASS) / LSS-A (GN) / LSS-B (SG)</v>
+        <v>SCM-C (RK) / LSS-B (SG)</v>
       </c>
       <c r="F74" t="str">
         <v/>
@@ -5356,7 +5356,7 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>2025-02-09</v>
+        <v>2025-02-02</v>
       </c>
       <c r="B75" t="str">
         <v>Sunday</v>
@@ -5371,7 +5371,7 @@
         <v/>
       </c>
       <c r="F75" t="str">
-        <v>GT (AG) / IPP (SRN)</v>
+        <v>GT (AG)</v>
       </c>
       <c r="G75" t="str">
         <v/>
@@ -5389,12 +5389,12 @@
         <v/>
       </c>
       <c r="L75" t="str">
-        <v/>
+        <v>SI-A (AK)</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>2025-02-09</v>
+        <v>2025-02-02</v>
       </c>
       <c r="B76" t="str">
         <v>Sunday</v>
@@ -5421,7 +5421,7 @@
         <v/>
       </c>
       <c r="J76" t="str">
-        <v>MBM (JT) / MMT (PN) / UOSWTPB (PS)</v>
+        <v>MBM (JT) / PBM-A (JJ)</v>
       </c>
       <c r="K76" t="str">
         <v/>
@@ -5432,7 +5432,7 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>2025-02-10</v>
+        <v>2025-02-03</v>
       </c>
       <c r="B77" t="str">
         <v>Monday</v>
@@ -5459,7 +5459,7 @@
         <v/>
       </c>
       <c r="J77" t="str">
-        <v>PBM-B (SS)</v>
+        <v>MBM (JT)</v>
       </c>
       <c r="K77" t="str">
         <v/>
@@ -5470,7 +5470,7 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>2025-02-11</v>
+        <v>2025-02-04</v>
       </c>
       <c r="B78" t="str">
         <v>Tuesday</v>
@@ -5508,7 +5508,7 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>2025-02-12</v>
+        <v>2025-02-05</v>
       </c>
       <c r="B79" t="str">
         <v>Wednesday</v>
@@ -5526,7 +5526,7 @@
         <v/>
       </c>
       <c r="G79" t="str">
-        <v>SAPM-A (ST) / ACF (ARS)</v>
+        <v/>
       </c>
       <c r="H79" t="str">
         <v/>
@@ -5546,10 +5546,10 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>2025-02-14</v>
+        <v>2025-02-06</v>
       </c>
       <c r="B80" t="str">
-        <v>Friday</v>
+        <v>Thursday</v>
       </c>
       <c r="C80" t="str">
         <v>19:00</v>
@@ -5558,16 +5558,16 @@
         <v>21:45</v>
       </c>
       <c r="E80" t="str">
-        <v>SCM-C (RK)</v>
+        <v/>
       </c>
       <c r="F80" t="str">
-        <v/>
+        <v>GT (AG) / ABMBM (VPV)</v>
       </c>
       <c r="G80" t="str">
         <v/>
       </c>
       <c r="H80" t="str">
-        <v>CCC (DS)</v>
+        <v/>
       </c>
       <c r="I80" t="str">
         <v/>
@@ -5584,19 +5584,19 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>2025-02-15</v>
+        <v>2025-02-07</v>
       </c>
       <c r="B81" t="str">
-        <v>Saturday</v>
+        <v>Friday</v>
       </c>
       <c r="C81" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D81" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E81" t="str">
-        <v/>
+        <v>LSS-A (GN) / LSS-B (SG)</v>
       </c>
       <c r="F81" t="str">
         <v/>
@@ -5605,7 +5605,7 @@
         <v/>
       </c>
       <c r="H81" t="str">
-        <v/>
+        <v>CCC (DS) / DPI (SAA)</v>
       </c>
       <c r="I81" t="str">
         <v/>
@@ -5614,7 +5614,7 @@
         <v/>
       </c>
       <c r="K81" t="str">
-        <v>LSO (PNR)</v>
+        <v/>
       </c>
       <c r="L81" t="str">
         <v/>
@@ -5622,16 +5622,16 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>2025-02-15</v>
+        <v>2025-02-08</v>
       </c>
       <c r="B82" t="str">
         <v>Saturday</v>
       </c>
       <c r="C82" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D82" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E82" t="str">
         <v/>
@@ -5640,7 +5640,7 @@
         <v/>
       </c>
       <c r="G82" t="str">
-        <v>SAPM-A (ST) / ACF (ARS)</v>
+        <v/>
       </c>
       <c r="H82" t="str">
         <v/>
@@ -5652,7 +5652,7 @@
         <v/>
       </c>
       <c r="K82" t="str">
-        <v/>
+        <v>LSO (PNR)</v>
       </c>
       <c r="L82" t="str">
         <v/>
@@ -5660,7 +5660,7 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>2025-02-16</v>
+        <v>2025-02-09</v>
       </c>
       <c r="B83" t="str">
         <v>Sunday</v>
@@ -5672,7 +5672,7 @@
         <v>11:45</v>
       </c>
       <c r="E83" t="str">
-        <v/>
+        <v>LSS-A (GN) / LSS-B (SG)</v>
       </c>
       <c r="F83" t="str">
         <v/>
@@ -5681,7 +5681,7 @@
         <v/>
       </c>
       <c r="H83" t="str">
-        <v>CCC (DS)</v>
+        <v>CCC (DS) / DPI (SAA)</v>
       </c>
       <c r="I83" t="str">
         <v/>
@@ -5698,22 +5698,22 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>2025-02-16</v>
+        <v>2025-02-09</v>
       </c>
       <c r="B84" t="str">
         <v>Sunday</v>
       </c>
       <c r="C84" t="str">
-        <v>15:30</v>
+        <v>12:15</v>
       </c>
       <c r="D84" t="str">
-        <v>18:15</v>
+        <v>15:00</v>
       </c>
       <c r="E84" t="str">
         <v/>
       </c>
       <c r="F84" t="str">
-        <v/>
+        <v>GT (AG) / ABMBM (VPV)</v>
       </c>
       <c r="G84" t="str">
         <v/>
@@ -5722,10 +5722,10 @@
         <v/>
       </c>
       <c r="I84" t="str">
-        <v>AIB-A (MPS)</v>
+        <v/>
       </c>
       <c r="J84" t="str">
-        <v>PBM-B (SS)</v>
+        <v/>
       </c>
       <c r="K84" t="str">
         <v/>
@@ -5736,10 +5736,10 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>2025-02-17</v>
+        <v>2025-02-09</v>
       </c>
       <c r="B85" t="str">
-        <v>Monday</v>
+        <v>Sunday</v>
       </c>
       <c r="C85" t="str">
         <v>15:30</v>
@@ -5760,10 +5760,10 @@
         <v/>
       </c>
       <c r="I85" t="str">
-        <v/>
+        <v>AIB-A (MPS)</v>
       </c>
       <c r="J85" t="str">
-        <v>SM (PB) / PBM-B (SS)</v>
+        <v>MBM (JT)</v>
       </c>
       <c r="K85" t="str">
         <v/>
@@ -5774,16 +5774,16 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>2025-02-18</v>
+        <v>2025-02-10</v>
       </c>
       <c r="B86" t="str">
-        <v>Tuesday</v>
+        <v>Monday</v>
       </c>
       <c r="C86" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D86" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E86" t="str">
         <v/>
@@ -5798,10 +5798,10 @@
         <v/>
       </c>
       <c r="I86" t="str">
-        <v>AIB-A (MPS)</v>
+        <v/>
       </c>
       <c r="J86" t="str">
-        <v/>
+        <v>SM (PB)</v>
       </c>
       <c r="K86" t="str">
         <v/>
@@ -5812,10 +5812,10 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>2025-02-19</v>
+        <v>2025-02-11</v>
       </c>
       <c r="B87" t="str">
-        <v>Wednesday</v>
+        <v>Tuesday</v>
       </c>
       <c r="C87" t="str">
         <v>19:00</v>
@@ -5830,19 +5830,19 @@
         <v/>
       </c>
       <c r="G87" t="str">
-        <v>PF (PKB)</v>
+        <v/>
       </c>
       <c r="H87" t="str">
         <v/>
       </c>
       <c r="I87" t="str">
-        <v/>
+        <v>AIB-A (MPS) / CSP (SRA)</v>
       </c>
       <c r="J87" t="str">
         <v/>
       </c>
       <c r="K87" t="str">
-        <v>LSO (PNR)</v>
+        <v/>
       </c>
       <c r="L87" t="str">
         <v/>
@@ -5850,10 +5850,10 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>2025-02-20</v>
+        <v>2025-02-12</v>
       </c>
       <c r="B88" t="str">
-        <v>Thursday</v>
+        <v>Wednesday</v>
       </c>
       <c r="C88" t="str">
         <v>19:00</v>
@@ -5865,10 +5865,10 @@
         <v/>
       </c>
       <c r="F88" t="str">
-        <v>GT (AG) / ABMBM (VPV)</v>
+        <v/>
       </c>
       <c r="G88" t="str">
-        <v/>
+        <v>ACF (ARS)</v>
       </c>
       <c r="H88" t="str">
         <v/>
@@ -5888,10 +5888,10 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>2025-02-21</v>
+        <v>2025-02-13</v>
       </c>
       <c r="B89" t="str">
-        <v>Friday</v>
+        <v>Thursday</v>
       </c>
       <c r="C89" t="str">
         <v>19:00</v>
@@ -5900,10 +5900,10 @@
         <v>21:45</v>
       </c>
       <c r="E89" t="str">
-        <v>LSS-B (SG)</v>
+        <v/>
       </c>
       <c r="F89" t="str">
-        <v/>
+        <v>ABMBM (VPV)</v>
       </c>
       <c r="G89" t="str">
         <v/>
@@ -5921,24 +5921,24 @@
         <v/>
       </c>
       <c r="L89" t="str">
-        <v/>
+        <v>MTI-B (AK)</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>2025-02-22</v>
+        <v>2025-02-14</v>
       </c>
       <c r="B90" t="str">
-        <v>Saturday</v>
+        <v>Friday</v>
       </c>
       <c r="C90" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D90" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E90" t="str">
-        <v/>
+        <v>SCM-B (SSP) / LSS-A (GN)</v>
       </c>
       <c r="F90" t="str">
         <v/>
@@ -5947,7 +5947,7 @@
         <v/>
       </c>
       <c r="H90" t="str">
-        <v/>
+        <v>ACCTP (DS)</v>
       </c>
       <c r="I90" t="str">
         <v/>
@@ -5956,7 +5956,7 @@
         <v/>
       </c>
       <c r="K90" t="str">
-        <v>LSO (PNR)</v>
+        <v/>
       </c>
       <c r="L90" t="str">
         <v/>
@@ -5964,7 +5964,7 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>2025-02-22</v>
+        <v>2025-02-15</v>
       </c>
       <c r="B91" t="str">
         <v>Saturday</v>
@@ -5982,7 +5982,7 @@
         <v/>
       </c>
       <c r="G91" t="str">
-        <v>PF (PKB)</v>
+        <v>ACF (ARS)</v>
       </c>
       <c r="H91" t="str">
         <v/>
@@ -6002,7 +6002,7 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>2025-02-23</v>
+        <v>2025-02-16</v>
       </c>
       <c r="B92" t="str">
         <v>Sunday</v>
@@ -6014,7 +6014,7 @@
         <v>11:45</v>
       </c>
       <c r="E92" t="str">
-        <v>LSS-B (SG)</v>
+        <v>SCM-B (SSP) / LSS-A (GN)</v>
       </c>
       <c r="F92" t="str">
         <v/>
@@ -6023,7 +6023,7 @@
         <v/>
       </c>
       <c r="H92" t="str">
-        <v/>
+        <v>ACCTP (DS)</v>
       </c>
       <c r="I92" t="str">
         <v/>
@@ -6040,7 +6040,7 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>2025-02-23</v>
+        <v>2025-02-16</v>
       </c>
       <c r="B93" t="str">
         <v>Sunday</v>
@@ -6055,7 +6055,7 @@
         <v/>
       </c>
       <c r="F93" t="str">
-        <v>GT (AG) / ABMBM (VPV)</v>
+        <v>ABMBM (VPV)</v>
       </c>
       <c r="G93" t="str">
         <v/>
@@ -6073,12 +6073,12 @@
         <v/>
       </c>
       <c r="L93" t="str">
-        <v/>
+        <v>MTI-B (AK)</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>2025-02-23</v>
+        <v>2025-02-16</v>
       </c>
       <c r="B94" t="str">
         <v>Sunday</v>
@@ -6102,10 +6102,10 @@
         <v/>
       </c>
       <c r="I94" t="str">
-        <v>AIB-A (MPS)</v>
+        <v>AIB-A (MPS) / CSP (SRA)</v>
       </c>
       <c r="J94" t="str">
-        <v>SM (PB) / PBM-B (SS)</v>
+        <v>SM (PB)</v>
       </c>
       <c r="K94" t="str">
         <v/>
@@ -6116,7 +6116,7 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>2025-02-24</v>
+        <v>2025-02-17</v>
       </c>
       <c r="B95" t="str">
         <v>Monday</v>
@@ -6143,7 +6143,7 @@
         <v/>
       </c>
       <c r="J95" t="str">
-        <v>SM (PB) / UOSWTPB (PS)</v>
+        <v>MBM (JT)</v>
       </c>
       <c r="K95" t="str">
         <v/>
@@ -6154,7 +6154,7 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>2025-02-25</v>
+        <v>2025-02-18</v>
       </c>
       <c r="B96" t="str">
         <v>Tuesday</v>
@@ -6178,7 +6178,7 @@
         <v/>
       </c>
       <c r="I96" t="str">
-        <v>CSP (SRA)</v>
+        <v>AIB-B (VK)</v>
       </c>
       <c r="J96" t="str">
         <v/>
@@ -6192,7 +6192,7 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>2025-02-26</v>
+        <v>2025-02-19</v>
       </c>
       <c r="B97" t="str">
         <v>Wednesday</v>
@@ -6210,7 +6210,7 @@
         <v/>
       </c>
       <c r="G97" t="str">
-        <v>SAPM-A (ST) / SAPM-B (VB) / ACF (ARS)</v>
+        <v>SAPM-B (VB) / PF (PKB)</v>
       </c>
       <c r="H97" t="str">
         <v/>
@@ -6230,7 +6230,7 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>2025-02-27</v>
+        <v>2025-02-20</v>
       </c>
       <c r="B98" t="str">
         <v>Thursday</v>
@@ -6245,7 +6245,7 @@
         <v/>
       </c>
       <c r="F98" t="str">
-        <v>GT (AG)</v>
+        <v/>
       </c>
       <c r="G98" t="str">
         <v/>
@@ -6263,12 +6263,12 @@
         <v/>
       </c>
       <c r="L98" t="str">
-        <v>SI-A (AK)</v>
+        <v>MTI-A (PV)</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>2025-02-28</v>
+        <v>2025-02-21</v>
       </c>
       <c r="B99" t="str">
         <v>Friday</v>
@@ -6280,7 +6280,7 @@
         <v>21:45</v>
       </c>
       <c r="E99" t="str">
-        <v>SCM-B (SSP) / SCM-C (RK)</v>
+        <v>SCM-A (ASS) / SCM-C (RK)</v>
       </c>
       <c r="F99" t="str">
         <v/>
@@ -6306,7 +6306,7 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>2025-03-01</v>
+        <v>2025-02-22</v>
       </c>
       <c r="B100" t="str">
         <v>Saturday</v>
@@ -6324,7 +6324,7 @@
         <v/>
       </c>
       <c r="G100" t="str">
-        <v>SAPM-A (ST) / SAPM-B (VB) / ACF (ARS)</v>
+        <v>SAPM-B (VB) / PF (PKB)</v>
       </c>
       <c r="H100" t="str">
         <v/>
@@ -6344,7 +6344,7 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>2025-03-02</v>
+        <v>2025-02-23</v>
       </c>
       <c r="B101" t="str">
         <v>Sunday</v>
@@ -6356,7 +6356,7 @@
         <v>11:45</v>
       </c>
       <c r="E101" t="str">
-        <v>SCM-B (SSP) / SCM-C (RK)</v>
+        <v>SCM-A (ASS) / SCM-C (RK)</v>
       </c>
       <c r="F101" t="str">
         <v/>
@@ -6365,7 +6365,7 @@
         <v/>
       </c>
       <c r="H101" t="str">
-        <v>CCC (DS)</v>
+        <v>ACCTP (DS)</v>
       </c>
       <c r="I101" t="str">
         <v/>
@@ -6382,7 +6382,7 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>2025-03-02</v>
+        <v>2025-02-23</v>
       </c>
       <c r="B102" t="str">
         <v>Sunday</v>
@@ -6397,7 +6397,7 @@
         <v/>
       </c>
       <c r="F102" t="str">
-        <v>GT (AG)</v>
+        <v/>
       </c>
       <c r="G102" t="str">
         <v/>
@@ -6415,12 +6415,12 @@
         <v/>
       </c>
       <c r="L102" t="str">
-        <v>SI-A (AK)</v>
+        <v>MTI-A (PV)</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>2025-03-02</v>
+        <v>2025-02-23</v>
       </c>
       <c r="B103" t="str">
         <v>Sunday</v>
@@ -6444,10 +6444,10 @@
         <v/>
       </c>
       <c r="I103" t="str">
-        <v>CSP (SRA)</v>
+        <v>AIB-B (VK)</v>
       </c>
       <c r="J103" t="str">
-        <v>SM (PB) / UOSWTPB (PS)</v>
+        <v>MBM (JT)</v>
       </c>
       <c r="K103" t="str">
         <v/>
@@ -6458,7 +6458,7 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>2025-03-03</v>
+        <v>2025-02-24</v>
       </c>
       <c r="B104" t="str">
         <v>Monday</v>
@@ -6485,7 +6485,7 @@
         <v/>
       </c>
       <c r="J104" t="str">
-        <v>SM (PB) / UOSWTPB (PS)</v>
+        <v>SM (PB) / PBM-A (JJ) / PBM-B (SS)</v>
       </c>
       <c r="K104" t="str">
         <v/>
@@ -6496,10 +6496,10 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>2025-03-04</v>
+        <v>2025-02-26</v>
       </c>
       <c r="B105" t="str">
-        <v>Tuesday</v>
+        <v>Wednesday</v>
       </c>
       <c r="C105" t="str">
         <v>19:00</v>
@@ -6514,19 +6514,19 @@
         <v/>
       </c>
       <c r="G105" t="str">
-        <v/>
+        <v>PF (PKB) / ACF (ARS)</v>
       </c>
       <c r="H105" t="str">
         <v/>
       </c>
       <c r="I105" t="str">
-        <v>AIB-B (VK)</v>
+        <v/>
       </c>
       <c r="J105" t="str">
         <v/>
       </c>
       <c r="K105" t="str">
-        <v/>
+        <v>LSO (PNR)</v>
       </c>
       <c r="L105" t="str">
         <v/>
@@ -6534,7 +6534,7 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>2025-03-06</v>
+        <v>2025-02-27</v>
       </c>
       <c r="B106" t="str">
         <v>Thursday</v>
@@ -6549,7 +6549,7 @@
         <v/>
       </c>
       <c r="F106" t="str">
-        <v>ABMBM (VPV)</v>
+        <v>GT (AG) / IPP (SRN)</v>
       </c>
       <c r="G106" t="str">
         <v/>
@@ -6567,12 +6567,12 @@
         <v/>
       </c>
       <c r="L106" t="str">
-        <v>MTI-B (AK)</v>
+        <v/>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>2025-03-07</v>
+        <v>2025-02-28</v>
       </c>
       <c r="B107" t="str">
         <v>Friday</v>
@@ -6584,7 +6584,7 @@
         <v>21:45</v>
       </c>
       <c r="E107" t="str">
-        <v>LSS-B (SG)</v>
+        <v>SCM-A (ASS) / SCM-C (RK)</v>
       </c>
       <c r="F107" t="str">
         <v/>
@@ -6593,7 +6593,7 @@
         <v/>
       </c>
       <c r="H107" t="str">
-        <v/>
+        <v>CCC (DS)</v>
       </c>
       <c r="I107" t="str">
         <v/>
@@ -6610,25 +6610,25 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>2025-03-09</v>
+        <v>2025-03-01</v>
       </c>
       <c r="B108" t="str">
-        <v>Sunday</v>
+        <v>Saturday</v>
       </c>
       <c r="C108" t="str">
-        <v>09:00</v>
+        <v>19:00</v>
       </c>
       <c r="D108" t="str">
-        <v>11:45</v>
+        <v>21:45</v>
       </c>
       <c r="E108" t="str">
-        <v>LSS-B (SG)</v>
+        <v/>
       </c>
       <c r="F108" t="str">
         <v/>
       </c>
       <c r="G108" t="str">
-        <v/>
+        <v>PF (PKB) / ACF (ARS)</v>
       </c>
       <c r="H108" t="str">
         <v/>
@@ -6648,28 +6648,28 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>2025-03-09</v>
+        <v>2025-03-02</v>
       </c>
       <c r="B109" t="str">
         <v>Sunday</v>
       </c>
       <c r="C109" t="str">
-        <v>12:15</v>
+        <v>09:00</v>
       </c>
       <c r="D109" t="str">
-        <v>15:00</v>
+        <v>11:45</v>
       </c>
       <c r="E109" t="str">
-        <v/>
+        <v>SCM-A (ASS) / SCM-C (RK)</v>
       </c>
       <c r="F109" t="str">
-        <v>ABMBM (VPV)</v>
+        <v/>
       </c>
       <c r="G109" t="str">
         <v/>
       </c>
       <c r="H109" t="str">
-        <v/>
+        <v>CCC (DS)</v>
       </c>
       <c r="I109" t="str">
         <v/>
@@ -6681,27 +6681,27 @@
         <v/>
       </c>
       <c r="L109" t="str">
-        <v>MTI-B (AK)</v>
+        <v/>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>2025-03-09</v>
+        <v>2025-03-02</v>
       </c>
       <c r="B110" t="str">
         <v>Sunday</v>
       </c>
       <c r="C110" t="str">
-        <v>15:30</v>
+        <v>12:15</v>
       </c>
       <c r="D110" t="str">
-        <v>18:15</v>
+        <v>15:00</v>
       </c>
       <c r="E110" t="str">
         <v/>
       </c>
       <c r="F110" t="str">
-        <v/>
+        <v>GT (AG) / IPP (SRN)</v>
       </c>
       <c r="G110" t="str">
         <v/>
@@ -6710,10 +6710,10 @@
         <v/>
       </c>
       <c r="I110" t="str">
-        <v>AIB-B (VK)</v>
+        <v/>
       </c>
       <c r="J110" t="str">
-        <v>SM (PB) / UOSWTPB (PS)</v>
+        <v/>
       </c>
       <c r="K110" t="str">
         <v/>
@@ -6724,22 +6724,22 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>2025-03-13</v>
+        <v>2025-03-02</v>
       </c>
       <c r="B111" t="str">
-        <v>Thursday</v>
+        <v>Sunday</v>
       </c>
       <c r="C111" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D111" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E111" t="str">
         <v/>
       </c>
       <c r="F111" t="str">
-        <v>ABMBM (VPV)</v>
+        <v/>
       </c>
       <c r="G111" t="str">
         <v/>
@@ -6751,30 +6751,30 @@
         <v/>
       </c>
       <c r="J111" t="str">
-        <v/>
+        <v>SM (PB) / PBM-A (JJ) / PBM-B (SS)</v>
       </c>
       <c r="K111" t="str">
         <v/>
       </c>
       <c r="L111" t="str">
-        <v>MASA (KKS)</v>
+        <v/>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>2025-03-14</v>
+        <v>2025-03-03</v>
       </c>
       <c r="B112" t="str">
-        <v>Friday</v>
+        <v>Monday</v>
       </c>
       <c r="C112" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D112" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E112" t="str">
-        <v>SCM-B (SSP) / LSS-A (GN)</v>
+        <v/>
       </c>
       <c r="F112" t="str">
         <v/>
@@ -6783,13 +6783,13 @@
         <v/>
       </c>
       <c r="H112" t="str">
-        <v>CCC (DS) / DPI (SAA)</v>
+        <v/>
       </c>
       <c r="I112" t="str">
         <v/>
       </c>
       <c r="J112" t="str">
-        <v/>
+        <v>PBM-B (SS) / MMT (PN) / UOSWTPB (PS)</v>
       </c>
       <c r="K112" t="str">
         <v/>
@@ -6800,16 +6800,16 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>2025-03-16</v>
+        <v>2025-03-04</v>
       </c>
       <c r="B113" t="str">
-        <v>Sunday</v>
+        <v>Tuesday</v>
       </c>
       <c r="C113" t="str">
-        <v>09:00</v>
+        <v>19:00</v>
       </c>
       <c r="D113" t="str">
-        <v>11:45</v>
+        <v>21:45</v>
       </c>
       <c r="E113" t="str">
         <v/>
@@ -6821,10 +6821,10 @@
         <v/>
       </c>
       <c r="H113" t="str">
-        <v>CCC (DS) / DPI (SAA)</v>
+        <v/>
       </c>
       <c r="I113" t="str">
-        <v/>
+        <v>CSP (SRA)</v>
       </c>
       <c r="J113" t="str">
         <v/>
@@ -6838,22 +6838,22 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>2025-03-16</v>
+        <v>2025-03-06</v>
       </c>
       <c r="B114" t="str">
-        <v>Sunday</v>
+        <v>Thursday</v>
       </c>
       <c r="C114" t="str">
-        <v>12:15</v>
+        <v>19:00</v>
       </c>
       <c r="D114" t="str">
-        <v>15:00</v>
+        <v>21:45</v>
       </c>
       <c r="E114" t="str">
         <v/>
       </c>
       <c r="F114" t="str">
-        <v>ABMBM (VPV)</v>
+        <v>GT (AG)</v>
       </c>
       <c r="G114" t="str">
         <v/>
@@ -6871,15 +6871,15 @@
         <v/>
       </c>
       <c r="L114" t="str">
-        <v>MASA (KKS)</v>
+        <v>MTI-A (PV)</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>2025-03-20</v>
+        <v>2025-03-07</v>
       </c>
       <c r="B115" t="str">
-        <v>Thursday</v>
+        <v>Friday</v>
       </c>
       <c r="C115" t="str">
         <v>19:00</v>
@@ -6888,7 +6888,7 @@
         <v>21:45</v>
       </c>
       <c r="E115" t="str">
-        <v/>
+        <v>SCM-A (ASS) / LSS-A (GN) / LSS-B (SG)</v>
       </c>
       <c r="F115" t="str">
         <v/>
@@ -6909,24 +6909,24 @@
         <v/>
       </c>
       <c r="L115" t="str">
-        <v>SI-B (PV) / MASA (KKS)</v>
+        <v/>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>2025-03-21</v>
+        <v>2025-03-09</v>
       </c>
       <c r="B116" t="str">
-        <v>Friday</v>
+        <v>Sunday</v>
       </c>
       <c r="C116" t="str">
-        <v>19:00</v>
+        <v>09:00</v>
       </c>
       <c r="D116" t="str">
-        <v>21:45</v>
+        <v>11:45</v>
       </c>
       <c r="E116" t="str">
-        <v/>
+        <v>SCM-A (ASS) / LSS-A (GN) / LSS-B (SG)</v>
       </c>
       <c r="F116" t="str">
         <v/>
@@ -6935,7 +6935,7 @@
         <v/>
       </c>
       <c r="H116" t="str">
-        <v>CCC (DS) / DPI (SAA)</v>
+        <v/>
       </c>
       <c r="I116" t="str">
         <v/>
@@ -6952,28 +6952,28 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>2025-03-23</v>
+        <v>2025-03-09</v>
       </c>
       <c r="B117" t="str">
         <v>Sunday</v>
       </c>
       <c r="C117" t="str">
-        <v>09:00</v>
+        <v>12:15</v>
       </c>
       <c r="D117" t="str">
-        <v>11:45</v>
+        <v>15:00</v>
       </c>
       <c r="E117" t="str">
         <v/>
       </c>
       <c r="F117" t="str">
-        <v/>
+        <v>GT (AG)</v>
       </c>
       <c r="G117" t="str">
         <v/>
       </c>
       <c r="H117" t="str">
-        <v>CCC (DS) / DPI (SAA)</v>
+        <v/>
       </c>
       <c r="I117" t="str">
         <v/>
@@ -6985,83 +6985,349 @@
         <v/>
       </c>
       <c r="L117" t="str">
-        <v/>
+        <v>MTI-A (PV)</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>2025-04-04</v>
+        <v>2025-03-09</v>
       </c>
       <c r="B118" t="str">
+        <v>Sunday</v>
+      </c>
+      <c r="C118" t="str">
+        <v>15:30</v>
+      </c>
+      <c r="D118" t="str">
+        <v>18:15</v>
+      </c>
+      <c r="E118" t="str">
+        <v/>
+      </c>
+      <c r="F118" t="str">
+        <v/>
+      </c>
+      <c r="G118" t="str">
+        <v/>
+      </c>
+      <c r="H118" t="str">
+        <v/>
+      </c>
+      <c r="I118" t="str">
+        <v>CSP (SRA)</v>
+      </c>
+      <c r="J118" t="str">
+        <v>PBM-B (SS) / MMT (PN) / UOSWTPB (PS)</v>
+      </c>
+      <c r="K118" t="str">
+        <v/>
+      </c>
+      <c r="L118" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>2025-03-13</v>
+      </c>
+      <c r="B119" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="C119" t="str">
+        <v>19:00</v>
+      </c>
+      <c r="D119" t="str">
+        <v>21:45</v>
+      </c>
+      <c r="E119" t="str">
+        <v/>
+      </c>
+      <c r="F119" t="str">
+        <v/>
+      </c>
+      <c r="G119" t="str">
+        <v/>
+      </c>
+      <c r="H119" t="str">
+        <v/>
+      </c>
+      <c r="I119" t="str">
+        <v/>
+      </c>
+      <c r="J119" t="str">
+        <v/>
+      </c>
+      <c r="K119" t="str">
+        <v/>
+      </c>
+      <c r="L119" t="str">
+        <v>SI-B (PV)</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>2025-03-14</v>
+      </c>
+      <c r="B120" t="str">
         <v>Friday</v>
       </c>
-      <c r="C118" t="str">
+      <c r="C120" t="str">
         <v>19:00</v>
       </c>
-      <c r="D118" t="str">
+      <c r="D120" t="str">
         <v>21:45</v>
       </c>
-      <c r="E118" t="str">
-        <v/>
-      </c>
-      <c r="F118" t="str">
-        <v/>
-      </c>
-      <c r="G118" t="str">
-        <v/>
-      </c>
-      <c r="H118" t="str">
+      <c r="E120" t="str">
+        <v/>
+      </c>
+      <c r="F120" t="str">
+        <v/>
+      </c>
+      <c r="G120" t="str">
+        <v/>
+      </c>
+      <c r="H120" t="str">
         <v>CCC (DS)</v>
       </c>
-      <c r="I118" t="str">
-        <v/>
-      </c>
-      <c r="J118" t="str">
-        <v/>
-      </c>
-      <c r="K118" t="str">
-        <v/>
-      </c>
-      <c r="L118" t="str">
+      <c r="I120" t="str">
+        <v/>
+      </c>
+      <c r="J120" t="str">
+        <v/>
+      </c>
+      <c r="K120" t="str">
+        <v/>
+      </c>
+      <c r="L120" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>2025-03-16</v>
+      </c>
+      <c r="B121" t="str">
+        <v>Sunday</v>
+      </c>
+      <c r="C121" t="str">
+        <v>09:00</v>
+      </c>
+      <c r="D121" t="str">
+        <v>11:45</v>
+      </c>
+      <c r="E121" t="str">
+        <v/>
+      </c>
+      <c r="F121" t="str">
+        <v/>
+      </c>
+      <c r="G121" t="str">
+        <v/>
+      </c>
+      <c r="H121" t="str">
+        <v>CCC (DS)</v>
+      </c>
+      <c r="I121" t="str">
+        <v/>
+      </c>
+      <c r="J121" t="str">
+        <v/>
+      </c>
+      <c r="K121" t="str">
+        <v/>
+      </c>
+      <c r="L121" t="str">
         <v/>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>__META__</v>
+        <v>2025-03-16</v>
       </c>
       <c r="B122" t="str">
-        <v>Generated At</v>
+        <v>Sunday</v>
       </c>
       <c r="C122" t="str">
-        <v>2026-05-27T17:59:42.833160</v>
+        <v>12:15</v>
+      </c>
+      <c r="D122" t="str">
+        <v>15:00</v>
+      </c>
+      <c r="E122" t="str">
+        <v/>
+      </c>
+      <c r="F122" t="str">
+        <v/>
+      </c>
+      <c r="G122" t="str">
+        <v/>
+      </c>
+      <c r="H122" t="str">
+        <v/>
+      </c>
+      <c r="I122" t="str">
+        <v/>
+      </c>
+      <c r="J122" t="str">
+        <v/>
+      </c>
+      <c r="K122" t="str">
+        <v/>
+      </c>
+      <c r="L122" t="str">
+        <v>SI-B (PV)</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>__META__</v>
+        <v>2025-03-21</v>
       </c>
       <c r="B123" t="str">
-        <v>Constraint</v>
+        <v>Friday</v>
       </c>
       <c r="C123" t="str">
-        <v>soft</v>
+        <v>19:00</v>
+      </c>
+      <c r="D123" t="str">
+        <v>21:45</v>
+      </c>
+      <c r="E123" t="str">
+        <v/>
+      </c>
+      <c r="F123" t="str">
+        <v/>
+      </c>
+      <c r="G123" t="str">
+        <v/>
+      </c>
+      <c r="H123" t="str">
+        <v>ACCTP (DS)</v>
+      </c>
+      <c r="I123" t="str">
+        <v/>
+      </c>
+      <c r="J123" t="str">
+        <v/>
+      </c>
+      <c r="K123" t="str">
+        <v/>
+      </c>
+      <c r="L123" t="str">
+        <v/>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
+        <v>2025-03-23</v>
+      </c>
+      <c r="B124" t="str">
+        <v>Sunday</v>
+      </c>
+      <c r="C124" t="str">
+        <v>15:30</v>
+      </c>
+      <c r="D124" t="str">
+        <v>18:15</v>
+      </c>
+      <c r="E124" t="str">
+        <v/>
+      </c>
+      <c r="F124" t="str">
+        <v/>
+      </c>
+      <c r="G124" t="str">
+        <v/>
+      </c>
+      <c r="H124" t="str">
+        <v/>
+      </c>
+      <c r="I124" t="str">
+        <v>AIB-B (VK)</v>
+      </c>
+      <c r="J124" t="str">
+        <v/>
+      </c>
+      <c r="K124" t="str">
+        <v/>
+      </c>
+      <c r="L124" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>2025-04-04</v>
+      </c>
+      <c r="B125" t="str">
+        <v>Friday</v>
+      </c>
+      <c r="C125" t="str">
+        <v>19:00</v>
+      </c>
+      <c r="D125" t="str">
+        <v>21:45</v>
+      </c>
+      <c r="E125" t="str">
+        <v/>
+      </c>
+      <c r="F125" t="str">
+        <v/>
+      </c>
+      <c r="G125" t="str">
+        <v/>
+      </c>
+      <c r="H125" t="str">
+        <v>ACCTP (DS) / DPI (SAA)</v>
+      </c>
+      <c r="I125" t="str">
+        <v/>
+      </c>
+      <c r="J125" t="str">
+        <v/>
+      </c>
+      <c r="K125" t="str">
+        <v/>
+      </c>
+      <c r="L125" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
         <v>__META__</v>
       </c>
-      <c r="B124" t="str">
+      <c r="B129" t="str">
+        <v>Generated At</v>
+      </c>
+      <c r="C129" t="str">
+        <v>2026-06-06T21:32:37.345551</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>__META__</v>
+      </c>
+      <c r="B130" t="str">
+        <v>Constraint</v>
+      </c>
+      <c r="C130" t="str">
+        <v>soft</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>__META__</v>
+      </c>
+      <c r="B131" t="str">
         <v>Penalty</v>
       </c>
-      <c r="C124">
+      <c r="C131">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L124"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L131"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added soft constraint on sessions spreading
</commit_message>
<xml_diff>
--- a/static/Areas_timetable_config.xlsx
+++ b/static/Areas_timetable_config.xlsx
@@ -420,7 +420,7 @@
         <v>Exported at</v>
       </c>
       <c r="B2" t="str">
-        <v>6/6/2026, 9:40:08 PM</v>
+        <v>6/26/2026, 10:15:23 PM</v>
       </c>
     </row>
     <row r="3">
@@ -2455,7 +2455,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -2517,16 +2517,32 @@
         <v>month</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>spreadingRule.enabled</v>
+      </c>
+      <c r="B8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>spreadingRule.weight</v>
+      </c>
+      <c r="B9">
+        <v>0.1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B9"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L131"/>
+  <dimension ref="A1:L121"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -2594,7 +2610,7 @@
         <v>11:45</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>LSS-A (GN) / SCM-B (SSP) / SCM-A (ASS)</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -2603,7 +2619,7 @@
         <v/>
       </c>
       <c r="H2" t="str">
-        <v>DPI (SAA)</v>
+        <v>CCC (DS)</v>
       </c>
       <c r="I2" t="str">
         <v/>
@@ -2626,16 +2642,16 @@
         <v>Sunday</v>
       </c>
       <c r="C3" t="str">
-        <v>15:30</v>
+        <v>12:15</v>
       </c>
       <c r="D3" t="str">
-        <v>18:15</v>
+        <v>15:00</v>
       </c>
       <c r="E3" t="str">
         <v/>
       </c>
       <c r="F3" t="str">
-        <v/>
+        <v>IPP (SRN)</v>
       </c>
       <c r="G3" t="str">
         <v/>
@@ -2644,24 +2660,24 @@
         <v/>
       </c>
       <c r="I3" t="str">
-        <v>AIB-B (VK)</v>
+        <v/>
       </c>
       <c r="J3" t="str">
-        <v>UOSWTPB (PS)</v>
+        <v/>
       </c>
       <c r="K3" t="str">
         <v/>
       </c>
       <c r="L3" t="str">
-        <v/>
+        <v>SI-A (AK) / SI-B (PV)</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2024-12-02</v>
+        <v>2024-12-01</v>
       </c>
       <c r="B4" t="str">
-        <v>Monday</v>
+        <v>Sunday</v>
       </c>
       <c r="C4" t="str">
         <v>15:30</v>
@@ -2682,10 +2698,10 @@
         <v/>
       </c>
       <c r="I4" t="str">
-        <v/>
+        <v>CSP (SRA)</v>
       </c>
       <c r="J4" t="str">
-        <v>PBM-B (SS)</v>
+        <v>MBM (JT) / SM (PB) / PBM-A (JJ)</v>
       </c>
       <c r="K4" t="str">
         <v/>
@@ -2696,16 +2712,16 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2024-12-03</v>
+        <v>2024-12-02</v>
       </c>
       <c r="B5" t="str">
-        <v>Tuesday</v>
+        <v>Monday</v>
       </c>
       <c r="C5" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D5" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E5" t="str">
         <v/>
@@ -2720,10 +2736,10 @@
         <v/>
       </c>
       <c r="I5" t="str">
-        <v>AIB-A (MPS) / CSP (SRA)</v>
+        <v/>
       </c>
       <c r="J5" t="str">
-        <v/>
+        <v>PBM-B (SS) / UOSWTPB (PS) / MMT (PN)</v>
       </c>
       <c r="K5" t="str">
         <v/>
@@ -2734,10 +2750,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2024-12-04</v>
+        <v>2024-12-03</v>
       </c>
       <c r="B6" t="str">
-        <v>Wednesday</v>
+        <v>Tuesday</v>
       </c>
       <c r="C6" t="str">
         <v>19:00</v>
@@ -2752,13 +2768,13 @@
         <v/>
       </c>
       <c r="G6" t="str">
-        <v>AMA (PKB) / SAPM-A (ST) / SAPM-B (VB)</v>
+        <v/>
       </c>
       <c r="H6" t="str">
         <v/>
       </c>
       <c r="I6" t="str">
-        <v/>
+        <v>AIB-B (VK)</v>
       </c>
       <c r="J6" t="str">
         <v/>
@@ -2772,10 +2788,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2024-12-05</v>
+        <v>2024-12-04</v>
       </c>
       <c r="B7" t="str">
-        <v>Thursday</v>
+        <v>Wednesday</v>
       </c>
       <c r="C7" t="str">
         <v>19:00</v>
@@ -2787,10 +2803,10 @@
         <v/>
       </c>
       <c r="F7" t="str">
-        <v>IPP (SRN)</v>
+        <v/>
       </c>
       <c r="G7" t="str">
-        <v/>
+        <v>SAPM-A (ST) / AMA (PKB)</v>
       </c>
       <c r="H7" t="str">
         <v/>
@@ -2802,18 +2818,18 @@
         <v/>
       </c>
       <c r="K7" t="str">
-        <v/>
+        <v>LSO (PNR)</v>
       </c>
       <c r="L7" t="str">
-        <v>SI-B (PV) / MASA (KKS)</v>
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2024-12-06</v>
+        <v>2024-12-05</v>
       </c>
       <c r="B8" t="str">
-        <v>Friday</v>
+        <v>Thursday</v>
       </c>
       <c r="C8" t="str">
         <v>19:00</v>
@@ -2822,10 +2838,10 @@
         <v>21:45</v>
       </c>
       <c r="E8" t="str">
-        <v>SCM-A (ASS) / LSS-B (SG)</v>
+        <v/>
       </c>
       <c r="F8" t="str">
-        <v/>
+        <v>GT (AG)</v>
       </c>
       <c r="G8" t="str">
         <v/>
@@ -2843,15 +2859,15 @@
         <v/>
       </c>
       <c r="L8" t="str">
-        <v/>
+        <v>MTI-A (PV)</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2024-12-07</v>
+        <v>2024-12-06</v>
       </c>
       <c r="B9" t="str">
-        <v>Saturday</v>
+        <v>Friday</v>
       </c>
       <c r="C9" t="str">
         <v>19:00</v>
@@ -2860,16 +2876,16 @@
         <v>21:45</v>
       </c>
       <c r="E9" t="str">
-        <v/>
+        <v>SCM-C (RK) / LSS-B (SG)</v>
       </c>
       <c r="F9" t="str">
         <v/>
       </c>
       <c r="G9" t="str">
-        <v>AMA (PKB) / SAPM-A (ST) / SAPM-B (VB)</v>
+        <v/>
       </c>
       <c r="H9" t="str">
-        <v/>
+        <v>ACCTP (DS) / DPI (SAA)</v>
       </c>
       <c r="I9" t="str">
         <v/>
@@ -2886,19 +2902,19 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2024-12-08</v>
+        <v>2024-12-07</v>
       </c>
       <c r="B10" t="str">
-        <v>Sunday</v>
+        <v>Saturday</v>
       </c>
       <c r="C10" t="str">
-        <v>09:00</v>
+        <v>15:30</v>
       </c>
       <c r="D10" t="str">
-        <v>11:45</v>
+        <v>18:15</v>
       </c>
       <c r="E10" t="str">
-        <v>SCM-A (ASS) / LSS-B (SG)</v>
+        <v/>
       </c>
       <c r="F10" t="str">
         <v/>
@@ -2916,7 +2932,7 @@
         <v/>
       </c>
       <c r="K10" t="str">
-        <v/>
+        <v>LSO (PNR)</v>
       </c>
       <c r="L10" t="str">
         <v/>
@@ -2924,25 +2940,25 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2024-12-08</v>
+        <v>2024-12-07</v>
       </c>
       <c r="B11" t="str">
-        <v>Sunday</v>
+        <v>Saturday</v>
       </c>
       <c r="C11" t="str">
-        <v>12:15</v>
+        <v>19:00</v>
       </c>
       <c r="D11" t="str">
-        <v>15:00</v>
+        <v>21:45</v>
       </c>
       <c r="E11" t="str">
         <v/>
       </c>
       <c r="F11" t="str">
-        <v>IPP (SRN)</v>
+        <v/>
       </c>
       <c r="G11" t="str">
-        <v/>
+        <v>ACF (ARS) / SAPM-A (ST)</v>
       </c>
       <c r="H11" t="str">
         <v/>
@@ -2957,7 +2973,7 @@
         <v/>
       </c>
       <c r="L11" t="str">
-        <v>SI-A (AK) / SI-B (PV) / MASA (KKS)</v>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -2968,13 +2984,13 @@
         <v>Sunday</v>
       </c>
       <c r="C12" t="str">
-        <v>15:30</v>
+        <v>09:00</v>
       </c>
       <c r="D12" t="str">
-        <v>18:15</v>
+        <v>11:45</v>
       </c>
       <c r="E12" t="str">
-        <v/>
+        <v>LSS-B (SG) / SCM-C (RK)</v>
       </c>
       <c r="F12" t="str">
         <v/>
@@ -2986,10 +3002,10 @@
         <v/>
       </c>
       <c r="I12" t="str">
-        <v>AIB-A (MPS) / CSP (SRA)</v>
+        <v/>
       </c>
       <c r="J12" t="str">
-        <v>PBM-B (SS)</v>
+        <v/>
       </c>
       <c r="K12" t="str">
         <v/>
@@ -3000,22 +3016,22 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2024-12-09</v>
+        <v>2024-12-08</v>
       </c>
       <c r="B13" t="str">
-        <v>Monday</v>
+        <v>Sunday</v>
       </c>
       <c r="C13" t="str">
-        <v>15:30</v>
+        <v>12:15</v>
       </c>
       <c r="D13" t="str">
-        <v>18:15</v>
+        <v>15:00</v>
       </c>
       <c r="E13" t="str">
         <v/>
       </c>
       <c r="F13" t="str">
-        <v/>
+        <v>GT (AG) / ABMBM (VPV)</v>
       </c>
       <c r="G13" t="str">
         <v/>
@@ -3027,27 +3043,27 @@
         <v/>
       </c>
       <c r="J13" t="str">
-        <v>MMT (PN)</v>
+        <v/>
       </c>
       <c r="K13" t="str">
         <v/>
       </c>
       <c r="L13" t="str">
-        <v/>
+        <v>MASA (KKS)</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2024-12-11</v>
+        <v>2024-12-08</v>
       </c>
       <c r="B14" t="str">
-        <v>Wednesday</v>
+        <v>Sunday</v>
       </c>
       <c r="C14" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D14" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E14" t="str">
         <v/>
@@ -3056,7 +3072,7 @@
         <v/>
       </c>
       <c r="G14" t="str">
-        <v>SAPM-A (ST)</v>
+        <v/>
       </c>
       <c r="H14" t="str">
         <v/>
@@ -3065,7 +3081,7 @@
         <v/>
       </c>
       <c r="J14" t="str">
-        <v/>
+        <v>UOSWTPB (PS)</v>
       </c>
       <c r="K14" t="str">
         <v/>
@@ -3076,16 +3092,16 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2024-12-12</v>
+        <v>2024-12-09</v>
       </c>
       <c r="B15" t="str">
-        <v>Thursday</v>
+        <v>Monday</v>
       </c>
       <c r="C15" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D15" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E15" t="str">
         <v/>
@@ -3103,21 +3119,21 @@
         <v/>
       </c>
       <c r="J15" t="str">
-        <v/>
+        <v>SM (PB) / MBM (JT)</v>
       </c>
       <c r="K15" t="str">
         <v/>
       </c>
       <c r="L15" t="str">
-        <v>MASA (KKS)</v>
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2024-12-13</v>
+        <v>2024-12-11</v>
       </c>
       <c r="B16" t="str">
-        <v>Friday</v>
+        <v>Wednesday</v>
       </c>
       <c r="C16" t="str">
         <v>19:00</v>
@@ -3132,10 +3148,10 @@
         <v/>
       </c>
       <c r="G16" t="str">
-        <v/>
+        <v>PF (PKB) / ACF (ARS)</v>
       </c>
       <c r="H16" t="str">
-        <v>CCC (DS)</v>
+        <v/>
       </c>
       <c r="I16" t="str">
         <v/>
@@ -3144,7 +3160,7 @@
         <v/>
       </c>
       <c r="K16" t="str">
-        <v/>
+        <v>LSO (PNR)</v>
       </c>
       <c r="L16" t="str">
         <v/>
@@ -3152,16 +3168,16 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2024-12-14</v>
+        <v>2024-12-12</v>
       </c>
       <c r="B17" t="str">
-        <v>Saturday</v>
+        <v>Thursday</v>
       </c>
       <c r="C17" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D17" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E17" t="str">
         <v/>
@@ -3182,18 +3198,18 @@
         <v/>
       </c>
       <c r="K17" t="str">
-        <v>LSO (PNR)</v>
+        <v/>
       </c>
       <c r="L17" t="str">
-        <v/>
+        <v>MTI-B (AK)</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2024-12-14</v>
+        <v>2024-12-13</v>
       </c>
       <c r="B18" t="str">
-        <v>Saturday</v>
+        <v>Friday</v>
       </c>
       <c r="C18" t="str">
         <v>19:00</v>
@@ -3202,16 +3218,16 @@
         <v>21:45</v>
       </c>
       <c r="E18" t="str">
-        <v/>
+        <v>LSS-A (GN)</v>
       </c>
       <c r="F18" t="str">
         <v/>
       </c>
       <c r="G18" t="str">
-        <v>SAPM-A (ST)</v>
+        <v/>
       </c>
       <c r="H18" t="str">
-        <v/>
+        <v>CCC (DS)</v>
       </c>
       <c r="I18" t="str">
         <v/>
@@ -3228,16 +3244,16 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2024-12-15</v>
+        <v>2024-12-14</v>
       </c>
       <c r="B19" t="str">
-        <v>Sunday</v>
+        <v>Saturday</v>
       </c>
       <c r="C19" t="str">
-        <v>12:15</v>
+        <v>19:00</v>
       </c>
       <c r="D19" t="str">
-        <v>15:00</v>
+        <v>21:45</v>
       </c>
       <c r="E19" t="str">
         <v/>
@@ -3246,7 +3262,7 @@
         <v/>
       </c>
       <c r="G19" t="str">
-        <v/>
+        <v>ACF (ARS) / PF (PKB) / SAPM-B (VB)</v>
       </c>
       <c r="H19" t="str">
         <v/>
@@ -3261,7 +3277,7 @@
         <v/>
       </c>
       <c r="L19" t="str">
-        <v>MASA (KKS)</v>
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -3272,13 +3288,13 @@
         <v>Sunday</v>
       </c>
       <c r="C20" t="str">
-        <v>15:30</v>
+        <v>09:00</v>
       </c>
       <c r="D20" t="str">
-        <v>18:15</v>
+        <v>11:45</v>
       </c>
       <c r="E20" t="str">
-        <v/>
+        <v>LSS-B (SG)</v>
       </c>
       <c r="F20" t="str">
         <v/>
@@ -3293,7 +3309,7 @@
         <v/>
       </c>
       <c r="J20" t="str">
-        <v>PBM-A (JJ) / MMT (PN)</v>
+        <v/>
       </c>
       <c r="K20" t="str">
         <v/>
@@ -3304,22 +3320,22 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2024-12-16</v>
+        <v>2024-12-15</v>
       </c>
       <c r="B21" t="str">
-        <v>Monday</v>
+        <v>Sunday</v>
       </c>
       <c r="C21" t="str">
-        <v>15:30</v>
+        <v>12:15</v>
       </c>
       <c r="D21" t="str">
-        <v>18:15</v>
+        <v>15:00</v>
       </c>
       <c r="E21" t="str">
         <v/>
       </c>
       <c r="F21" t="str">
-        <v/>
+        <v>GT (AG)</v>
       </c>
       <c r="G21" t="str">
         <v/>
@@ -3331,7 +3347,7 @@
         <v/>
       </c>
       <c r="J21" t="str">
-        <v>SM (PB) / PBM-A (JJ) / PBM-B (SS)</v>
+        <v/>
       </c>
       <c r="K21" t="str">
         <v/>
@@ -3342,16 +3358,16 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2024-12-18</v>
+        <v>2024-12-15</v>
       </c>
       <c r="B22" t="str">
-        <v>Wednesday</v>
+        <v>Sunday</v>
       </c>
       <c r="C22" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D22" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E22" t="str">
         <v/>
@@ -3360,16 +3376,16 @@
         <v/>
       </c>
       <c r="G22" t="str">
-        <v>SAPM-B (VB) / ACF (ARS)</v>
+        <v/>
       </c>
       <c r="H22" t="str">
         <v/>
       </c>
       <c r="I22" t="str">
-        <v/>
+        <v>AIB-A (MPS)</v>
       </c>
       <c r="J22" t="str">
-        <v/>
+        <v>MBM (JT)</v>
       </c>
       <c r="K22" t="str">
         <v/>
@@ -3380,16 +3396,16 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2024-12-21</v>
+        <v>2024-12-23</v>
       </c>
       <c r="B23" t="str">
-        <v>Saturday</v>
+        <v>Monday</v>
       </c>
       <c r="C23" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D23" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E23" t="str">
         <v/>
@@ -3398,7 +3414,7 @@
         <v/>
       </c>
       <c r="G23" t="str">
-        <v>SAPM-B (VB) / ACF (ARS)</v>
+        <v/>
       </c>
       <c r="H23" t="str">
         <v/>
@@ -3407,7 +3423,7 @@
         <v/>
       </c>
       <c r="J23" t="str">
-        <v/>
+        <v>MMT (PN) / PBM-B (SS) / UOSWTPB (PS)</v>
       </c>
       <c r="K23" t="str">
         <v/>
@@ -3418,16 +3434,16 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2024-12-22</v>
+        <v>2024-12-24</v>
       </c>
       <c r="B24" t="str">
-        <v>Sunday</v>
+        <v>Tuesday</v>
       </c>
       <c r="C24" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D24" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E24" t="str">
         <v/>
@@ -3442,10 +3458,10 @@
         <v/>
       </c>
       <c r="I24" t="str">
-        <v/>
+        <v>CSP (SRA) / AIB-A (MPS)</v>
       </c>
       <c r="J24" t="str">
-        <v>SM (PB) / PBM-B (SS)</v>
+        <v/>
       </c>
       <c r="K24" t="str">
         <v/>
@@ -3456,16 +3472,16 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2024-12-23</v>
+        <v>2024-12-25</v>
       </c>
       <c r="B25" t="str">
-        <v>Monday</v>
+        <v>Wednesday</v>
       </c>
       <c r="C25" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D25" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E25" t="str">
         <v/>
@@ -3483,10 +3499,10 @@
         <v/>
       </c>
       <c r="J25" t="str">
-        <v>MBM (JT)</v>
+        <v/>
       </c>
       <c r="K25" t="str">
-        <v/>
+        <v>LSO (PNR)</v>
       </c>
       <c r="L25" t="str">
         <v/>
@@ -3494,10 +3510,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2024-12-24</v>
+        <v>2024-12-26</v>
       </c>
       <c r="B26" t="str">
-        <v>Tuesday</v>
+        <v>Thursday</v>
       </c>
       <c r="C26" t="str">
         <v>19:00</v>
@@ -3509,7 +3525,7 @@
         <v/>
       </c>
       <c r="F26" t="str">
-        <v/>
+        <v>IPP (SRN) / GT (AG)</v>
       </c>
       <c r="G26" t="str">
         <v/>
@@ -3518,7 +3534,7 @@
         <v/>
       </c>
       <c r="I26" t="str">
-        <v>AIB-A (MPS)</v>
+        <v/>
       </c>
       <c r="J26" t="str">
         <v/>
@@ -3527,15 +3543,15 @@
         <v/>
       </c>
       <c r="L26" t="str">
-        <v/>
+        <v>MASA (KKS)</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2024-12-25</v>
+        <v>2024-12-27</v>
       </c>
       <c r="B27" t="str">
-        <v>Wednesday</v>
+        <v>Friday</v>
       </c>
       <c r="C27" t="str">
         <v>19:00</v>
@@ -3544,16 +3560,16 @@
         <v>21:45</v>
       </c>
       <c r="E27" t="str">
-        <v/>
+        <v>SCM-B (SSP) / SCM-C (RK)</v>
       </c>
       <c r="F27" t="str">
         <v/>
       </c>
       <c r="G27" t="str">
-        <v>PF (PKB)</v>
+        <v/>
       </c>
       <c r="H27" t="str">
-        <v/>
+        <v>CCC (DS) / DPI (SAA)</v>
       </c>
       <c r="I27" t="str">
         <v/>
@@ -3570,10 +3586,10 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2024-12-27</v>
+        <v>2024-12-28</v>
       </c>
       <c r="B28" t="str">
-        <v>Friday</v>
+        <v>Saturday</v>
       </c>
       <c r="C28" t="str">
         <v>19:00</v>
@@ -3582,13 +3598,13 @@
         <v>21:45</v>
       </c>
       <c r="E28" t="str">
-        <v>SCM-B (SSP) / SCM-C (RK)</v>
+        <v/>
       </c>
       <c r="F28" t="str">
         <v/>
       </c>
       <c r="G28" t="str">
-        <v/>
+        <v>SAPM-A (ST)</v>
       </c>
       <c r="H28" t="str">
         <v/>
@@ -3608,28 +3624,28 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2024-12-28</v>
+        <v>2024-12-29</v>
       </c>
       <c r="B29" t="str">
-        <v>Saturday</v>
+        <v>Sunday</v>
       </c>
       <c r="C29" t="str">
-        <v>19:00</v>
+        <v>09:00</v>
       </c>
       <c r="D29" t="str">
-        <v>21:45</v>
+        <v>11:45</v>
       </c>
       <c r="E29" t="str">
-        <v/>
+        <v>LSS-A (GN) / LSS-B (SG) / SCM-A (ASS)</v>
       </c>
       <c r="F29" t="str">
         <v/>
       </c>
       <c r="G29" t="str">
-        <v>PF (PKB)</v>
+        <v/>
       </c>
       <c r="H29" t="str">
-        <v/>
+        <v>ACCTP (DS)</v>
       </c>
       <c r="I29" t="str">
         <v/>
@@ -3652,16 +3668,16 @@
         <v>Sunday</v>
       </c>
       <c r="C30" t="str">
-        <v>09:00</v>
+        <v>12:15</v>
       </c>
       <c r="D30" t="str">
-        <v>11:45</v>
+        <v>15:00</v>
       </c>
       <c r="E30" t="str">
-        <v>SCM-B (SSP) / SCM-C (RK)</v>
+        <v/>
       </c>
       <c r="F30" t="str">
-        <v/>
+        <v>ABMBM (VPV)</v>
       </c>
       <c r="G30" t="str">
         <v/>
@@ -3679,7 +3695,7 @@
         <v/>
       </c>
       <c r="L30" t="str">
-        <v/>
+        <v>MASA (KKS)</v>
       </c>
     </row>
     <row r="31">
@@ -3708,7 +3724,7 @@
         <v/>
       </c>
       <c r="I31" t="str">
-        <v>AIB-A (MPS)</v>
+        <v/>
       </c>
       <c r="J31" t="str">
         <v>MBM (JT)</v>
@@ -3749,7 +3765,7 @@
         <v/>
       </c>
       <c r="J32" t="str">
-        <v>UOSWTPB (PS)</v>
+        <v>SM (PB) / PBM-A (JJ) / PBM-B (SS)</v>
       </c>
       <c r="K32" t="str">
         <v/>
@@ -3760,10 +3776,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2025-01-01</v>
+        <v>2024-12-31</v>
       </c>
       <c r="B33" t="str">
-        <v>Wednesday</v>
+        <v>Tuesday</v>
       </c>
       <c r="C33" t="str">
         <v>19:00</v>
@@ -3778,13 +3794,13 @@
         <v/>
       </c>
       <c r="G33" t="str">
-        <v>ACF (ARS)</v>
+        <v/>
       </c>
       <c r="H33" t="str">
         <v/>
       </c>
       <c r="I33" t="str">
-        <v/>
+        <v>AIB-B (VK)</v>
       </c>
       <c r="J33" t="str">
         <v/>
@@ -3798,10 +3814,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2025-01-02</v>
+        <v>2025-01-01</v>
       </c>
       <c r="B34" t="str">
-        <v>Thursday</v>
+        <v>Wednesday</v>
       </c>
       <c r="C34" t="str">
         <v>19:00</v>
@@ -3813,10 +3829,10 @@
         <v/>
       </c>
       <c r="F34" t="str">
-        <v>GT (AG)</v>
+        <v/>
       </c>
       <c r="G34" t="str">
-        <v/>
+        <v>PF (PKB) / SAPM-B (VB) / ACF (ARS)</v>
       </c>
       <c r="H34" t="str">
         <v/>
@@ -3836,10 +3852,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2025-01-03</v>
+        <v>2025-01-02</v>
       </c>
       <c r="B35" t="str">
-        <v>Friday</v>
+        <v>Thursday</v>
       </c>
       <c r="C35" t="str">
         <v>19:00</v>
@@ -3848,7 +3864,7 @@
         <v>21:45</v>
       </c>
       <c r="E35" t="str">
-        <v>SCM-B (SSP) / LSS-A (GN)</v>
+        <v/>
       </c>
       <c r="F35" t="str">
         <v/>
@@ -3857,7 +3873,7 @@
         <v/>
       </c>
       <c r="H35" t="str">
-        <v>CCC (DS)</v>
+        <v/>
       </c>
       <c r="I35" t="str">
         <v/>
@@ -3869,15 +3885,15 @@
         <v/>
       </c>
       <c r="L35" t="str">
-        <v/>
+        <v>SI-B (PV)</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2025-01-04</v>
+        <v>2025-01-03</v>
       </c>
       <c r="B36" t="str">
-        <v>Saturday</v>
+        <v>Friday</v>
       </c>
       <c r="C36" t="str">
         <v>19:00</v>
@@ -3886,16 +3902,16 @@
         <v>21:45</v>
       </c>
       <c r="E36" t="str">
-        <v/>
+        <v>LSS-A (GN) / SCM-B (SSP) / SCM-A (ASS)</v>
       </c>
       <c r="F36" t="str">
         <v/>
       </c>
       <c r="G36" t="str">
-        <v>ACF (ARS)</v>
+        <v/>
       </c>
       <c r="H36" t="str">
-        <v/>
+        <v>ACCTP (DS)</v>
       </c>
       <c r="I36" t="str">
         <v/>
@@ -3912,28 +3928,28 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>2025-01-05</v>
+        <v>2025-01-04</v>
       </c>
       <c r="B37" t="str">
-        <v>Sunday</v>
+        <v>Saturday</v>
       </c>
       <c r="C37" t="str">
-        <v>09:00</v>
+        <v>19:00</v>
       </c>
       <c r="D37" t="str">
-        <v>11:45</v>
+        <v>21:45</v>
       </c>
       <c r="E37" t="str">
-        <v>SCM-B (SSP) / LSS-A (GN)</v>
+        <v/>
       </c>
       <c r="F37" t="str">
         <v/>
       </c>
       <c r="G37" t="str">
-        <v/>
+        <v>PF (PKB) / ACF (ARS)</v>
       </c>
       <c r="H37" t="str">
-        <v>CCC (DS)</v>
+        <v/>
       </c>
       <c r="I37" t="str">
         <v/>
@@ -3956,16 +3972,16 @@
         <v>Sunday</v>
       </c>
       <c r="C38" t="str">
-        <v>12:15</v>
+        <v>09:00</v>
       </c>
       <c r="D38" t="str">
-        <v>15:00</v>
+        <v>11:45</v>
       </c>
       <c r="E38" t="str">
-        <v/>
+        <v>SCM-B (SSP) / SCM-C (RK) / SCM-A (ASS)</v>
       </c>
       <c r="F38" t="str">
-        <v>GT (AG)</v>
+        <v/>
       </c>
       <c r="G38" t="str">
         <v/>
@@ -3983,7 +3999,7 @@
         <v/>
       </c>
       <c r="L38" t="str">
-        <v>SI-A (AK)</v>
+        <v/>
       </c>
     </row>
     <row r="39">
@@ -3994,16 +4010,16 @@
         <v>Sunday</v>
       </c>
       <c r="C39" t="str">
-        <v>15:30</v>
+        <v>12:15</v>
       </c>
       <c r="D39" t="str">
-        <v>18:15</v>
+        <v>15:00</v>
       </c>
       <c r="E39" t="str">
         <v/>
       </c>
       <c r="F39" t="str">
-        <v/>
+        <v>IPP (SRN)</v>
       </c>
       <c r="G39" t="str">
         <v/>
@@ -4015,21 +4031,21 @@
         <v/>
       </c>
       <c r="J39" t="str">
-        <v>UOSWTPB (PS)</v>
+        <v/>
       </c>
       <c r="K39" t="str">
         <v/>
       </c>
       <c r="L39" t="str">
-        <v/>
+        <v>MTI-A (PV)</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>2025-01-06</v>
+        <v>2025-01-05</v>
       </c>
       <c r="B40" t="str">
-        <v>Monday</v>
+        <v>Sunday</v>
       </c>
       <c r="C40" t="str">
         <v>15:30</v>
@@ -4050,10 +4066,10 @@
         <v/>
       </c>
       <c r="I40" t="str">
-        <v/>
+        <v>AIB-B (VK)</v>
       </c>
       <c r="J40" t="str">
-        <v>MBM (JT) / PBM-A (JJ) / MMT (PN)</v>
+        <v>PBM-B (SS) / SM (PB) / PBM-A (JJ)</v>
       </c>
       <c r="K40" t="str">
         <v/>
@@ -4064,16 +4080,16 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>2025-01-07</v>
+        <v>2025-01-06</v>
       </c>
       <c r="B41" t="str">
-        <v>Tuesday</v>
+        <v>Monday</v>
       </c>
       <c r="C41" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D41" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E41" t="str">
         <v/>
@@ -4088,10 +4104,10 @@
         <v/>
       </c>
       <c r="I41" t="str">
-        <v>AIB-B (VK)</v>
+        <v/>
       </c>
       <c r="J41" t="str">
-        <v/>
+        <v>UOSWTPB (PS) / MBM (JT) / MMT (PN)</v>
       </c>
       <c r="K41" t="str">
         <v/>
@@ -4102,10 +4118,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>2025-01-08</v>
+        <v>2025-01-07</v>
       </c>
       <c r="B42" t="str">
-        <v>Wednesday</v>
+        <v>Tuesday</v>
       </c>
       <c r="C42" t="str">
         <v>19:00</v>
@@ -4120,19 +4136,19 @@
         <v/>
       </c>
       <c r="G42" t="str">
-        <v>SAPM-A (ST) / ACF (ARS)</v>
+        <v/>
       </c>
       <c r="H42" t="str">
         <v/>
       </c>
       <c r="I42" t="str">
-        <v/>
+        <v>CSP (SRA)</v>
       </c>
       <c r="J42" t="str">
         <v/>
       </c>
       <c r="K42" t="str">
-        <v>LSO (PNR)</v>
+        <v/>
       </c>
       <c r="L42" t="str">
         <v/>
@@ -4140,10 +4156,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>2025-01-09</v>
+        <v>2025-01-08</v>
       </c>
       <c r="B43" t="str">
-        <v>Thursday</v>
+        <v>Wednesday</v>
       </c>
       <c r="C43" t="str">
         <v>19:00</v>
@@ -4155,10 +4171,10 @@
         <v/>
       </c>
       <c r="F43" t="str">
-        <v>IPP (SRN)</v>
+        <v/>
       </c>
       <c r="G43" t="str">
-        <v/>
+        <v>ACF (ARS) / SAPM-B (VB) / SAPM-A (ST)</v>
       </c>
       <c r="H43" t="str">
         <v/>
@@ -4173,15 +4189,15 @@
         <v/>
       </c>
       <c r="L43" t="str">
-        <v>MTI-B (AK) / MASA (KKS)</v>
+        <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>2025-01-10</v>
+        <v>2025-01-09</v>
       </c>
       <c r="B44" t="str">
-        <v>Friday</v>
+        <v>Thursday</v>
       </c>
       <c r="C44" t="str">
         <v>19:00</v>
@@ -4190,16 +4206,16 @@
         <v>21:45</v>
       </c>
       <c r="E44" t="str">
-        <v>LSS-A (GN) / LSS-B (SG)</v>
+        <v/>
       </c>
       <c r="F44" t="str">
-        <v/>
+        <v>GT (AG) / ABMBM (VPV)</v>
       </c>
       <c r="G44" t="str">
         <v/>
       </c>
       <c r="H44" t="str">
-        <v>CCC (DS)</v>
+        <v/>
       </c>
       <c r="I44" t="str">
         <v/>
@@ -4211,24 +4227,24 @@
         <v/>
       </c>
       <c r="L44" t="str">
-        <v/>
+        <v>MASA (KKS)</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>2025-01-11</v>
+        <v>2025-01-10</v>
       </c>
       <c r="B45" t="str">
-        <v>Saturday</v>
+        <v>Friday</v>
       </c>
       <c r="C45" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D45" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E45" t="str">
-        <v/>
+        <v>LSS-B (SG) / LSS-A (GN)</v>
       </c>
       <c r="F45" t="str">
         <v/>
@@ -4237,7 +4253,7 @@
         <v/>
       </c>
       <c r="H45" t="str">
-        <v/>
+        <v>CCC (DS)</v>
       </c>
       <c r="I45" t="str">
         <v/>
@@ -4246,7 +4262,7 @@
         <v/>
       </c>
       <c r="K45" t="str">
-        <v>LSO (PNR)</v>
+        <v/>
       </c>
       <c r="L45" t="str">
         <v/>
@@ -4272,7 +4288,7 @@
         <v/>
       </c>
       <c r="G46" t="str">
-        <v>SAPM-A (ST) / ACF (ARS)</v>
+        <v>AMA (PKB)</v>
       </c>
       <c r="H46" t="str">
         <v/>
@@ -4313,7 +4329,7 @@
         <v/>
       </c>
       <c r="H47" t="str">
-        <v>CCC (DS)</v>
+        <v>DPI (SAA) / CCC (DS)</v>
       </c>
       <c r="I47" t="str">
         <v/>
@@ -4345,7 +4361,7 @@
         <v/>
       </c>
       <c r="F48" t="str">
-        <v>IPP (SRN)</v>
+        <v>GT (AG)</v>
       </c>
       <c r="G48" t="str">
         <v/>
@@ -4363,7 +4379,7 @@
         <v/>
       </c>
       <c r="L48" t="str">
-        <v>MTI-B (AK) / MASA (KKS)</v>
+        <v>SI-A (AK)</v>
       </c>
     </row>
     <row r="49">
@@ -4392,10 +4408,10 @@
         <v/>
       </c>
       <c r="I49" t="str">
-        <v>AIB-B (VK)</v>
+        <v>AIB-A (MPS)</v>
       </c>
       <c r="J49" t="str">
-        <v>MBM (JT) / PBM-A (JJ) / MMT (PN)</v>
+        <v>MMT (PN) / MBM (JT)</v>
       </c>
       <c r="K49" t="str">
         <v/>
@@ -4406,16 +4422,16 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>2025-01-13</v>
+        <v>2025-01-15</v>
       </c>
       <c r="B50" t="str">
-        <v>Monday</v>
+        <v>Wednesday</v>
       </c>
       <c r="C50" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D50" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E50" t="str">
         <v/>
@@ -4424,7 +4440,7 @@
         <v/>
       </c>
       <c r="G50" t="str">
-        <v/>
+        <v>PF (PKB)</v>
       </c>
       <c r="H50" t="str">
         <v/>
@@ -4433,10 +4449,10 @@
         <v/>
       </c>
       <c r="J50" t="str">
-        <v>SM (PB) / UOSWTPB (PS)</v>
+        <v/>
       </c>
       <c r="K50" t="str">
-        <v/>
+        <v>LSO (PNR)</v>
       </c>
       <c r="L50" t="str">
         <v/>
@@ -4444,10 +4460,10 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>2025-01-14</v>
+        <v>2025-01-17</v>
       </c>
       <c r="B51" t="str">
-        <v>Tuesday</v>
+        <v>Friday</v>
       </c>
       <c r="C51" t="str">
         <v>19:00</v>
@@ -4456,7 +4472,7 @@
         <v>21:45</v>
       </c>
       <c r="E51" t="str">
-        <v/>
+        <v>SCM-A (ASS) / SCM-B (SSP) / SCM-C (RK)</v>
       </c>
       <c r="F51" t="str">
         <v/>
@@ -4468,7 +4484,7 @@
         <v/>
       </c>
       <c r="I51" t="str">
-        <v>CSP (SRA)</v>
+        <v/>
       </c>
       <c r="J51" t="str">
         <v/>
@@ -4482,10 +4498,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>2025-01-15</v>
+        <v>2025-01-18</v>
       </c>
       <c r="B52" t="str">
-        <v>Wednesday</v>
+        <v>Saturday</v>
       </c>
       <c r="C52" t="str">
         <v>19:00</v>
@@ -4500,7 +4516,7 @@
         <v/>
       </c>
       <c r="G52" t="str">
-        <v>AMA (PKB) / SAPM-A (ST) / SAPM-B (VB)</v>
+        <v>PF (PKB)</v>
       </c>
       <c r="H52" t="str">
         <v/>
@@ -4520,22 +4536,22 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>2025-01-16</v>
+        <v>2025-01-20</v>
       </c>
       <c r="B53" t="str">
-        <v>Thursday</v>
+        <v>Monday</v>
       </c>
       <c r="C53" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D53" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E53" t="str">
         <v/>
       </c>
       <c r="F53" t="str">
-        <v>GT (AG) / IPP (SRN) / ABMBM (VPV)</v>
+        <v/>
       </c>
       <c r="G53" t="str">
         <v/>
@@ -4547,21 +4563,21 @@
         <v/>
       </c>
       <c r="J53" t="str">
-        <v/>
+        <v>MBM (JT) / PBM-A (JJ)</v>
       </c>
       <c r="K53" t="str">
         <v/>
       </c>
       <c r="L53" t="str">
-        <v>MASA (KKS)</v>
+        <v/>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>2025-01-17</v>
+        <v>2025-01-21</v>
       </c>
       <c r="B54" t="str">
-        <v>Friday</v>
+        <v>Tuesday</v>
       </c>
       <c r="C54" t="str">
         <v>19:00</v>
@@ -4570,7 +4586,7 @@
         <v>21:45</v>
       </c>
       <c r="E54" t="str">
-        <v>SCM-B (SSP)</v>
+        <v/>
       </c>
       <c r="F54" t="str">
         <v/>
@@ -4579,10 +4595,10 @@
         <v/>
       </c>
       <c r="H54" t="str">
-        <v>DPI (SAA)</v>
+        <v/>
       </c>
       <c r="I54" t="str">
-        <v/>
+        <v>AIB-B (VK)</v>
       </c>
       <c r="J54" t="str">
         <v/>
@@ -4596,10 +4612,10 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>2025-01-18</v>
+        <v>2025-01-22</v>
       </c>
       <c r="B55" t="str">
-        <v>Saturday</v>
+        <v>Wednesday</v>
       </c>
       <c r="C55" t="str">
         <v>19:00</v>
@@ -4614,7 +4630,7 @@
         <v/>
       </c>
       <c r="G55" t="str">
-        <v>AMA (PKB) / SAPM-A (ST) / SAPM-B (VB)</v>
+        <v>SAPM-B (VB) / ACF (ARS)</v>
       </c>
       <c r="H55" t="str">
         <v/>
@@ -4634,28 +4650,28 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>2025-01-19</v>
+        <v>2025-01-23</v>
       </c>
       <c r="B56" t="str">
-        <v>Sunday</v>
+        <v>Thursday</v>
       </c>
       <c r="C56" t="str">
-        <v>09:00</v>
+        <v>19:00</v>
       </c>
       <c r="D56" t="str">
-        <v>11:45</v>
+        <v>21:45</v>
       </c>
       <c r="E56" t="str">
-        <v>SCM-B (SSP)</v>
+        <v/>
       </c>
       <c r="F56" t="str">
-        <v/>
+        <v>GT (AG) / IPP (SRN)</v>
       </c>
       <c r="G56" t="str">
         <v/>
       </c>
       <c r="H56" t="str">
-        <v>DPI (SAA)</v>
+        <v/>
       </c>
       <c r="I56" t="str">
         <v/>
@@ -4672,28 +4688,28 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>2025-01-19</v>
+        <v>2025-01-24</v>
       </c>
       <c r="B57" t="str">
-        <v>Sunday</v>
+        <v>Friday</v>
       </c>
       <c r="C57" t="str">
-        <v>12:15</v>
+        <v>19:00</v>
       </c>
       <c r="D57" t="str">
-        <v>15:00</v>
+        <v>21:45</v>
       </c>
       <c r="E57" t="str">
         <v/>
       </c>
       <c r="F57" t="str">
-        <v>GT (AG) / IPP (SRN) / ABMBM (VPV)</v>
+        <v/>
       </c>
       <c r="G57" t="str">
         <v/>
       </c>
       <c r="H57" t="str">
-        <v/>
+        <v>ACCTP (DS)</v>
       </c>
       <c r="I57" t="str">
         <v/>
@@ -4705,21 +4721,21 @@
         <v/>
       </c>
       <c r="L57" t="str">
-        <v>MASA (KKS)</v>
+        <v/>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>2025-01-19</v>
+        <v>2025-01-25</v>
       </c>
       <c r="B58" t="str">
-        <v>Sunday</v>
+        <v>Saturday</v>
       </c>
       <c r="C58" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D58" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E58" t="str">
         <v/>
@@ -4728,16 +4744,16 @@
         <v/>
       </c>
       <c r="G58" t="str">
-        <v/>
+        <v>ACF (ARS)</v>
       </c>
       <c r="H58" t="str">
         <v/>
       </c>
       <c r="I58" t="str">
-        <v>CSP (SRA)</v>
+        <v/>
       </c>
       <c r="J58" t="str">
-        <v>SM (PB) / UOSWTPB (PS)</v>
+        <v/>
       </c>
       <c r="K58" t="str">
         <v/>
@@ -4748,10 +4764,10 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>2025-01-20</v>
+        <v>2025-01-26</v>
       </c>
       <c r="B59" t="str">
-        <v>Monday</v>
+        <v>Sunday</v>
       </c>
       <c r="C59" t="str">
         <v>15:30</v>
@@ -4772,10 +4788,10 @@
         <v/>
       </c>
       <c r="I59" t="str">
-        <v/>
+        <v>AIB-A (MPS)</v>
       </c>
       <c r="J59" t="str">
-        <v>MBM (JT) / MMT (PN)</v>
+        <v>MMT (PN) / MBM (JT)</v>
       </c>
       <c r="K59" t="str">
         <v/>
@@ -4786,16 +4802,16 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>2025-01-21</v>
+        <v>2025-01-27</v>
       </c>
       <c r="B60" t="str">
-        <v>Tuesday</v>
+        <v>Monday</v>
       </c>
       <c r="C60" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D60" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E60" t="str">
         <v/>
@@ -4810,10 +4826,10 @@
         <v/>
       </c>
       <c r="I60" t="str">
-        <v>AIB-B (VK)</v>
+        <v/>
       </c>
       <c r="J60" t="str">
-        <v/>
+        <v>PBM-B (SS) / UOSWTPB (PS) / SM (PB)</v>
       </c>
       <c r="K60" t="str">
         <v/>
@@ -4824,10 +4840,10 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>2025-01-22</v>
+        <v>2025-01-28</v>
       </c>
       <c r="B61" t="str">
-        <v>Wednesday</v>
+        <v>Tuesday</v>
       </c>
       <c r="C61" t="str">
         <v>19:00</v>
@@ -4842,13 +4858,13 @@
         <v/>
       </c>
       <c r="G61" t="str">
-        <v>PF (PKB) / ACF (ARS)</v>
+        <v/>
       </c>
       <c r="H61" t="str">
         <v/>
       </c>
       <c r="I61" t="str">
-        <v/>
+        <v>CSP (SRA)</v>
       </c>
       <c r="J61" t="str">
         <v/>
@@ -4862,10 +4878,10 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>2025-01-23</v>
+        <v>2025-01-29</v>
       </c>
       <c r="B62" t="str">
-        <v>Thursday</v>
+        <v>Wednesday</v>
       </c>
       <c r="C62" t="str">
         <v>19:00</v>
@@ -4877,10 +4893,10 @@
         <v/>
       </c>
       <c r="F62" t="str">
-        <v>ABMBM (VPV)</v>
+        <v/>
       </c>
       <c r="G62" t="str">
-        <v/>
+        <v>SAPM-B (VB) / SAPM-A (ST) / AMA (PKB)</v>
       </c>
       <c r="H62" t="str">
         <v/>
@@ -4900,10 +4916,10 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>2025-01-24</v>
+        <v>2025-01-30</v>
       </c>
       <c r="B63" t="str">
-        <v>Friday</v>
+        <v>Thursday</v>
       </c>
       <c r="C63" t="str">
         <v>19:00</v>
@@ -4912,16 +4928,16 @@
         <v>21:45</v>
       </c>
       <c r="E63" t="str">
-        <v>LSS-A (GN) / LSS-B (SG)</v>
+        <v/>
       </c>
       <c r="F63" t="str">
-        <v/>
+        <v>ABMBM (VPV)</v>
       </c>
       <c r="G63" t="str">
         <v/>
       </c>
       <c r="H63" t="str">
-        <v>ACCTP (DS) / DPI (SAA)</v>
+        <v/>
       </c>
       <c r="I63" t="str">
         <v/>
@@ -4933,15 +4949,15 @@
         <v/>
       </c>
       <c r="L63" t="str">
-        <v/>
+        <v>MASA (KKS) / MTI-B (AK)</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>2025-01-25</v>
+        <v>2025-01-31</v>
       </c>
       <c r="B64" t="str">
-        <v>Saturday</v>
+        <v>Friday</v>
       </c>
       <c r="C64" t="str">
         <v>19:00</v>
@@ -4950,16 +4966,16 @@
         <v>21:45</v>
       </c>
       <c r="E64" t="str">
-        <v/>
+        <v>LSS-A (GN) / LSS-B (SG)</v>
       </c>
       <c r="F64" t="str">
         <v/>
       </c>
       <c r="G64" t="str">
-        <v>PF (PKB) / ACF (ARS)</v>
+        <v/>
       </c>
       <c r="H64" t="str">
-        <v/>
+        <v>DPI (SAA) / CCC (DS)</v>
       </c>
       <c r="I64" t="str">
         <v/>
@@ -4976,19 +4992,19 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>2025-01-26</v>
+        <v>2025-02-01</v>
       </c>
       <c r="B65" t="str">
-        <v>Sunday</v>
+        <v>Saturday</v>
       </c>
       <c r="C65" t="str">
-        <v>09:00</v>
+        <v>15:30</v>
       </c>
       <c r="D65" t="str">
-        <v>11:45</v>
+        <v>18:15</v>
       </c>
       <c r="E65" t="str">
-        <v>LSS-A (GN) / LSS-B (SG)</v>
+        <v/>
       </c>
       <c r="F65" t="str">
         <v/>
@@ -4997,7 +5013,7 @@
         <v/>
       </c>
       <c r="H65" t="str">
-        <v>ACCTP (DS) / DPI (SAA)</v>
+        <v/>
       </c>
       <c r="I65" t="str">
         <v/>
@@ -5006,7 +5022,7 @@
         <v/>
       </c>
       <c r="K65" t="str">
-        <v/>
+        <v>LSO (PNR)</v>
       </c>
       <c r="L65" t="str">
         <v/>
@@ -5014,25 +5030,25 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>2025-01-26</v>
+        <v>2025-02-01</v>
       </c>
       <c r="B66" t="str">
-        <v>Sunday</v>
+        <v>Saturday</v>
       </c>
       <c r="C66" t="str">
-        <v>12:15</v>
+        <v>19:00</v>
       </c>
       <c r="D66" t="str">
-        <v>15:00</v>
+        <v>21:45</v>
       </c>
       <c r="E66" t="str">
         <v/>
       </c>
       <c r="F66" t="str">
-        <v>ABMBM (VPV)</v>
+        <v/>
       </c>
       <c r="G66" t="str">
-        <v/>
+        <v>AMA (PKB) / SAPM-A (ST)</v>
       </c>
       <c r="H66" t="str">
         <v/>
@@ -5052,19 +5068,19 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>2025-01-26</v>
+        <v>2025-02-02</v>
       </c>
       <c r="B67" t="str">
         <v>Sunday</v>
       </c>
       <c r="C67" t="str">
-        <v>15:30</v>
+        <v>09:00</v>
       </c>
       <c r="D67" t="str">
-        <v>18:15</v>
+        <v>11:45</v>
       </c>
       <c r="E67" t="str">
-        <v/>
+        <v>LSS-B (SG) / LSS-A (GN)</v>
       </c>
       <c r="F67" t="str">
         <v/>
@@ -5076,10 +5092,10 @@
         <v/>
       </c>
       <c r="I67" t="str">
-        <v>AIB-B (VK)</v>
+        <v/>
       </c>
       <c r="J67" t="str">
-        <v>MBM (JT) / MMT (PN) / UOSWTPB (PS)</v>
+        <v/>
       </c>
       <c r="K67" t="str">
         <v/>
@@ -5090,22 +5106,22 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>2025-01-27</v>
+        <v>2025-02-02</v>
       </c>
       <c r="B68" t="str">
-        <v>Monday</v>
+        <v>Sunday</v>
       </c>
       <c r="C68" t="str">
-        <v>15:30</v>
+        <v>12:15</v>
       </c>
       <c r="D68" t="str">
-        <v>18:15</v>
+        <v>15:00</v>
       </c>
       <c r="E68" t="str">
         <v/>
       </c>
       <c r="F68" t="str">
-        <v/>
+        <v>ABMBM (VPV)</v>
       </c>
       <c r="G68" t="str">
         <v/>
@@ -5117,27 +5133,27 @@
         <v/>
       </c>
       <c r="J68" t="str">
-        <v>MBM (JT) / PBM-A (JJ)</v>
+        <v/>
       </c>
       <c r="K68" t="str">
         <v/>
       </c>
       <c r="L68" t="str">
-        <v/>
+        <v>MTI-B (AK) / MASA (KKS)</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>2025-01-29</v>
+        <v>2025-02-02</v>
       </c>
       <c r="B69" t="str">
-        <v>Wednesday</v>
+        <v>Sunday</v>
       </c>
       <c r="C69" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D69" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E69" t="str">
         <v/>
@@ -5146,19 +5162,19 @@
         <v/>
       </c>
       <c r="G69" t="str">
-        <v>AMA (PKB)</v>
+        <v/>
       </c>
       <c r="H69" t="str">
         <v/>
       </c>
       <c r="I69" t="str">
-        <v/>
+        <v>CSP (SRA) / AIB-A (MPS)</v>
       </c>
       <c r="J69" t="str">
-        <v/>
+        <v>SM (PB) / PBM-B (SS)</v>
       </c>
       <c r="K69" t="str">
-        <v>LSO (PNR)</v>
+        <v/>
       </c>
       <c r="L69" t="str">
         <v/>
@@ -5166,22 +5182,22 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>2025-01-30</v>
+        <v>2025-02-03</v>
       </c>
       <c r="B70" t="str">
-        <v>Thursday</v>
+        <v>Monday</v>
       </c>
       <c r="C70" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D70" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E70" t="str">
         <v/>
       </c>
       <c r="F70" t="str">
-        <v>GT (AG)</v>
+        <v/>
       </c>
       <c r="G70" t="str">
         <v/>
@@ -5193,21 +5209,21 @@
         <v/>
       </c>
       <c r="J70" t="str">
-        <v/>
+        <v>MMT (PN) / MBM (JT) / PBM-A (JJ)</v>
       </c>
       <c r="K70" t="str">
         <v/>
       </c>
       <c r="L70" t="str">
-        <v>SI-A (AK)</v>
+        <v/>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>2025-01-31</v>
+        <v>2025-02-04</v>
       </c>
       <c r="B71" t="str">
-        <v>Friday</v>
+        <v>Tuesday</v>
       </c>
       <c r="C71" t="str">
         <v>19:00</v>
@@ -5216,7 +5232,7 @@
         <v>21:45</v>
       </c>
       <c r="E71" t="str">
-        <v>SCM-C (RK) / LSS-B (SG)</v>
+        <v/>
       </c>
       <c r="F71" t="str">
         <v/>
@@ -5225,10 +5241,10 @@
         <v/>
       </c>
       <c r="H71" t="str">
-        <v>CCC (DS)</v>
+        <v/>
       </c>
       <c r="I71" t="str">
-        <v/>
+        <v>AIB-B (VK)</v>
       </c>
       <c r="J71" t="str">
         <v/>
@@ -5242,16 +5258,16 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>2025-02-01</v>
+        <v>2025-02-05</v>
       </c>
       <c r="B72" t="str">
-        <v>Saturday</v>
+        <v>Wednesday</v>
       </c>
       <c r="C72" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D72" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E72" t="str">
         <v/>
@@ -5260,7 +5276,7 @@
         <v/>
       </c>
       <c r="G72" t="str">
-        <v/>
+        <v>ACF (ARS) / PF (PKB)</v>
       </c>
       <c r="H72" t="str">
         <v/>
@@ -5280,10 +5296,10 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>2025-02-01</v>
+        <v>2025-02-06</v>
       </c>
       <c r="B73" t="str">
-        <v>Saturday</v>
+        <v>Thursday</v>
       </c>
       <c r="C73" t="str">
         <v>19:00</v>
@@ -5295,10 +5311,10 @@
         <v/>
       </c>
       <c r="F73" t="str">
-        <v/>
+        <v>GT (AG) / IPP (SRN)</v>
       </c>
       <c r="G73" t="str">
-        <v>AMA (PKB)</v>
+        <v/>
       </c>
       <c r="H73" t="str">
         <v/>
@@ -5313,24 +5329,24 @@
         <v/>
       </c>
       <c r="L73" t="str">
-        <v/>
+        <v>MTI-A (PV)</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>2025-02-02</v>
+        <v>2025-02-07</v>
       </c>
       <c r="B74" t="str">
-        <v>Sunday</v>
+        <v>Friday</v>
       </c>
       <c r="C74" t="str">
-        <v>09:00</v>
+        <v>19:00</v>
       </c>
       <c r="D74" t="str">
-        <v>11:45</v>
+        <v>21:45</v>
       </c>
       <c r="E74" t="str">
-        <v>SCM-C (RK) / LSS-B (SG)</v>
+        <v>SCM-B (SSP) / SCM-C (RK) / SCM-A (ASS)</v>
       </c>
       <c r="F74" t="str">
         <v/>
@@ -5339,7 +5355,7 @@
         <v/>
       </c>
       <c r="H74" t="str">
-        <v/>
+        <v>ACCTP (DS)</v>
       </c>
       <c r="I74" t="str">
         <v/>
@@ -5356,25 +5372,25 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>2025-02-02</v>
+        <v>2025-02-08</v>
       </c>
       <c r="B75" t="str">
-        <v>Sunday</v>
+        <v>Saturday</v>
       </c>
       <c r="C75" t="str">
-        <v>12:15</v>
+        <v>19:00</v>
       </c>
       <c r="D75" t="str">
-        <v>15:00</v>
+        <v>21:45</v>
       </c>
       <c r="E75" t="str">
         <v/>
       </c>
       <c r="F75" t="str">
-        <v>GT (AG)</v>
+        <v/>
       </c>
       <c r="G75" t="str">
-        <v/>
+        <v>AMA (PKB) / SAPM-A (ST)</v>
       </c>
       <c r="H75" t="str">
         <v/>
@@ -5389,21 +5405,21 @@
         <v/>
       </c>
       <c r="L75" t="str">
-        <v>SI-A (AK)</v>
+        <v/>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>2025-02-02</v>
+        <v>2025-02-09</v>
       </c>
       <c r="B76" t="str">
         <v>Sunday</v>
       </c>
       <c r="C76" t="str">
-        <v>15:30</v>
+        <v>09:00</v>
       </c>
       <c r="D76" t="str">
-        <v>18:15</v>
+        <v>11:45</v>
       </c>
       <c r="E76" t="str">
         <v/>
@@ -5415,13 +5431,13 @@
         <v/>
       </c>
       <c r="H76" t="str">
-        <v/>
+        <v>DPI (SAA) / CCC (DS)</v>
       </c>
       <c r="I76" t="str">
         <v/>
       </c>
       <c r="J76" t="str">
-        <v>MBM (JT) / PBM-A (JJ)</v>
+        <v/>
       </c>
       <c r="K76" t="str">
         <v/>
@@ -5432,16 +5448,16 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>2025-02-03</v>
+        <v>2025-02-09</v>
       </c>
       <c r="B77" t="str">
-        <v>Monday</v>
+        <v>Sunday</v>
       </c>
       <c r="C77" t="str">
-        <v>15:30</v>
+        <v>12:15</v>
       </c>
       <c r="D77" t="str">
-        <v>18:15</v>
+        <v>15:00</v>
       </c>
       <c r="E77" t="str">
         <v/>
@@ -5459,27 +5475,27 @@
         <v/>
       </c>
       <c r="J77" t="str">
-        <v>MBM (JT)</v>
+        <v/>
       </c>
       <c r="K77" t="str">
         <v/>
       </c>
       <c r="L77" t="str">
-        <v/>
+        <v>SI-B (PV)</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>2025-02-04</v>
+        <v>2025-02-09</v>
       </c>
       <c r="B78" t="str">
-        <v>Tuesday</v>
+        <v>Sunday</v>
       </c>
       <c r="C78" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D78" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E78" t="str">
         <v/>
@@ -5494,10 +5510,10 @@
         <v/>
       </c>
       <c r="I78" t="str">
-        <v>AIB-A (MPS)</v>
+        <v/>
       </c>
       <c r="J78" t="str">
-        <v/>
+        <v>UOSWTPB (PS) / MBM (JT)</v>
       </c>
       <c r="K78" t="str">
         <v/>
@@ -5508,7 +5524,7 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>2025-02-05</v>
+        <v>2025-02-12</v>
       </c>
       <c r="B79" t="str">
         <v>Wednesday</v>
@@ -5526,7 +5542,7 @@
         <v/>
       </c>
       <c r="G79" t="str">
-        <v/>
+        <v>SAPM-B (VB) / ACF (ARS)</v>
       </c>
       <c r="H79" t="str">
         <v/>
@@ -5538,7 +5554,7 @@
         <v/>
       </c>
       <c r="K79" t="str">
-        <v>LSO (PNR)</v>
+        <v/>
       </c>
       <c r="L79" t="str">
         <v/>
@@ -5546,7 +5562,7 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>2025-02-06</v>
+        <v>2025-02-13</v>
       </c>
       <c r="B80" t="str">
         <v>Thursday</v>
@@ -5561,7 +5577,7 @@
         <v/>
       </c>
       <c r="F80" t="str">
-        <v>GT (AG) / ABMBM (VPV)</v>
+        <v>GT (AG)</v>
       </c>
       <c r="G80" t="str">
         <v/>
@@ -5584,7 +5600,7 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>2025-02-07</v>
+        <v>2025-02-14</v>
       </c>
       <c r="B81" t="str">
         <v>Friday</v>
@@ -5596,7 +5612,7 @@
         <v>21:45</v>
       </c>
       <c r="E81" t="str">
-        <v>LSS-A (GN) / LSS-B (SG)</v>
+        <v>LSS-B (SG)</v>
       </c>
       <c r="F81" t="str">
         <v/>
@@ -5605,7 +5621,7 @@
         <v/>
       </c>
       <c r="H81" t="str">
-        <v>CCC (DS) / DPI (SAA)</v>
+        <v>CCC (DS)</v>
       </c>
       <c r="I81" t="str">
         <v/>
@@ -5622,16 +5638,16 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>2025-02-08</v>
+        <v>2025-02-15</v>
       </c>
       <c r="B82" t="str">
         <v>Saturday</v>
       </c>
       <c r="C82" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D82" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E82" t="str">
         <v/>
@@ -5640,7 +5656,7 @@
         <v/>
       </c>
       <c r="G82" t="str">
-        <v/>
+        <v>ACF (ARS)</v>
       </c>
       <c r="H82" t="str">
         <v/>
@@ -5652,7 +5668,7 @@
         <v/>
       </c>
       <c r="K82" t="str">
-        <v>LSO (PNR)</v>
+        <v/>
       </c>
       <c r="L82" t="str">
         <v/>
@@ -5660,19 +5676,19 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>2025-02-09</v>
+        <v>2025-02-17</v>
       </c>
       <c r="B83" t="str">
-        <v>Sunday</v>
+        <v>Monday</v>
       </c>
       <c r="C83" t="str">
-        <v>09:00</v>
+        <v>15:30</v>
       </c>
       <c r="D83" t="str">
-        <v>11:45</v>
+        <v>18:15</v>
       </c>
       <c r="E83" t="str">
-        <v>LSS-A (GN) / LSS-B (SG)</v>
+        <v/>
       </c>
       <c r="F83" t="str">
         <v/>
@@ -5681,13 +5697,13 @@
         <v/>
       </c>
       <c r="H83" t="str">
-        <v>CCC (DS) / DPI (SAA)</v>
+        <v/>
       </c>
       <c r="I83" t="str">
         <v/>
       </c>
       <c r="J83" t="str">
-        <v/>
+        <v>SM (PB) / UOSWTPB (PS) / MBM (JT)</v>
       </c>
       <c r="K83" t="str">
         <v/>
@@ -5698,25 +5714,25 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>2025-02-09</v>
+        <v>2025-02-19</v>
       </c>
       <c r="B84" t="str">
-        <v>Sunday</v>
+        <v>Wednesday</v>
       </c>
       <c r="C84" t="str">
-        <v>12:15</v>
+        <v>19:00</v>
       </c>
       <c r="D84" t="str">
-        <v>15:00</v>
+        <v>21:45</v>
       </c>
       <c r="E84" t="str">
         <v/>
       </c>
       <c r="F84" t="str">
-        <v>GT (AG) / ABMBM (VPV)</v>
+        <v/>
       </c>
       <c r="G84" t="str">
-        <v/>
+        <v>PF (PKB)</v>
       </c>
       <c r="H84" t="str">
         <v/>
@@ -5728,7 +5744,7 @@
         <v/>
       </c>
       <c r="K84" t="str">
-        <v/>
+        <v>LSO (PNR)</v>
       </c>
       <c r="L84" t="str">
         <v/>
@@ -5736,22 +5752,22 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>2025-02-09</v>
+        <v>2025-02-20</v>
       </c>
       <c r="B85" t="str">
-        <v>Sunday</v>
+        <v>Thursday</v>
       </c>
       <c r="C85" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D85" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E85" t="str">
         <v/>
       </c>
       <c r="F85" t="str">
-        <v/>
+        <v>IPP (SRN)</v>
       </c>
       <c r="G85" t="str">
         <v/>
@@ -5760,10 +5776,10 @@
         <v/>
       </c>
       <c r="I85" t="str">
-        <v>AIB-A (MPS)</v>
+        <v/>
       </c>
       <c r="J85" t="str">
-        <v>MBM (JT)</v>
+        <v/>
       </c>
       <c r="K85" t="str">
         <v/>
@@ -5774,19 +5790,19 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>2025-02-10</v>
+        <v>2025-02-21</v>
       </c>
       <c r="B86" t="str">
-        <v>Monday</v>
+        <v>Friday</v>
       </c>
       <c r="C86" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D86" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E86" t="str">
-        <v/>
+        <v>LSS-A (GN) / SCM-A (ASS) / SCM-B (SSP)</v>
       </c>
       <c r="F86" t="str">
         <v/>
@@ -5795,13 +5811,13 @@
         <v/>
       </c>
       <c r="H86" t="str">
-        <v/>
+        <v>ACCTP (DS)</v>
       </c>
       <c r="I86" t="str">
         <v/>
       </c>
       <c r="J86" t="str">
-        <v>SM (PB)</v>
+        <v/>
       </c>
       <c r="K86" t="str">
         <v/>
@@ -5812,19 +5828,19 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>2025-02-11</v>
+        <v>2025-02-23</v>
       </c>
       <c r="B87" t="str">
-        <v>Tuesday</v>
+        <v>Sunday</v>
       </c>
       <c r="C87" t="str">
-        <v>19:00</v>
+        <v>09:00</v>
       </c>
       <c r="D87" t="str">
-        <v>21:45</v>
+        <v>11:45</v>
       </c>
       <c r="E87" t="str">
-        <v/>
+        <v>LSS-A (GN)</v>
       </c>
       <c r="F87" t="str">
         <v/>
@@ -5836,7 +5852,7 @@
         <v/>
       </c>
       <c r="I87" t="str">
-        <v>AIB-A (MPS) / CSP (SRA)</v>
+        <v/>
       </c>
       <c r="J87" t="str">
         <v/>
@@ -5850,16 +5866,16 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>2025-02-12</v>
+        <v>2025-02-23</v>
       </c>
       <c r="B88" t="str">
-        <v>Wednesday</v>
+        <v>Sunday</v>
       </c>
       <c r="C88" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D88" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E88" t="str">
         <v/>
@@ -5868,7 +5884,7 @@
         <v/>
       </c>
       <c r="G88" t="str">
-        <v>ACF (ARS)</v>
+        <v/>
       </c>
       <c r="H88" t="str">
         <v/>
@@ -5877,7 +5893,7 @@
         <v/>
       </c>
       <c r="J88" t="str">
-        <v/>
+        <v>UOSWTPB (PS) / MBM (JT) / SM (PB)</v>
       </c>
       <c r="K88" t="str">
         <v/>
@@ -5888,22 +5904,22 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>2025-02-13</v>
+        <v>2025-02-24</v>
       </c>
       <c r="B89" t="str">
-        <v>Thursday</v>
+        <v>Monday</v>
       </c>
       <c r="C89" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D89" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E89" t="str">
         <v/>
       </c>
       <c r="F89" t="str">
-        <v>ABMBM (VPV)</v>
+        <v/>
       </c>
       <c r="G89" t="str">
         <v/>
@@ -5915,21 +5931,21 @@
         <v/>
       </c>
       <c r="J89" t="str">
-        <v/>
+        <v>PBM-A (JJ) / MMT (PN) / PBM-B (SS)</v>
       </c>
       <c r="K89" t="str">
         <v/>
       </c>
       <c r="L89" t="str">
-        <v>MTI-B (AK)</v>
+        <v/>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>2025-02-14</v>
+        <v>2025-02-25</v>
       </c>
       <c r="B90" t="str">
-        <v>Friday</v>
+        <v>Tuesday</v>
       </c>
       <c r="C90" t="str">
         <v>19:00</v>
@@ -5938,7 +5954,7 @@
         <v>21:45</v>
       </c>
       <c r="E90" t="str">
-        <v>SCM-B (SSP) / LSS-A (GN)</v>
+        <v/>
       </c>
       <c r="F90" t="str">
         <v/>
@@ -5947,10 +5963,10 @@
         <v/>
       </c>
       <c r="H90" t="str">
-        <v>ACCTP (DS)</v>
+        <v/>
       </c>
       <c r="I90" t="str">
-        <v/>
+        <v>AIB-B (VK)</v>
       </c>
       <c r="J90" t="str">
         <v/>
@@ -5964,10 +5980,10 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>2025-02-15</v>
+        <v>2025-02-26</v>
       </c>
       <c r="B91" t="str">
-        <v>Saturday</v>
+        <v>Wednesday</v>
       </c>
       <c r="C91" t="str">
         <v>19:00</v>
@@ -5982,7 +5998,7 @@
         <v/>
       </c>
       <c r="G91" t="str">
-        <v>ACF (ARS)</v>
+        <v>ACF (ARS) / SAPM-B (VB) / SAPM-A (ST)</v>
       </c>
       <c r="H91" t="str">
         <v/>
@@ -6002,28 +6018,28 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>2025-02-16</v>
+        <v>2025-02-27</v>
       </c>
       <c r="B92" t="str">
-        <v>Sunday</v>
+        <v>Thursday</v>
       </c>
       <c r="C92" t="str">
-        <v>09:00</v>
+        <v>19:00</v>
       </c>
       <c r="D92" t="str">
-        <v>11:45</v>
+        <v>21:45</v>
       </c>
       <c r="E92" t="str">
-        <v>SCM-B (SSP) / LSS-A (GN)</v>
+        <v/>
       </c>
       <c r="F92" t="str">
-        <v/>
+        <v>GT (AG)</v>
       </c>
       <c r="G92" t="str">
         <v/>
       </c>
       <c r="H92" t="str">
-        <v>ACCTP (DS)</v>
+        <v/>
       </c>
       <c r="I92" t="str">
         <v/>
@@ -6035,33 +6051,33 @@
         <v/>
       </c>
       <c r="L92" t="str">
-        <v/>
+        <v>SI-A (AK) / MASA (KKS)</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>2025-02-16</v>
+        <v>2025-02-28</v>
       </c>
       <c r="B93" t="str">
-        <v>Sunday</v>
+        <v>Friday</v>
       </c>
       <c r="C93" t="str">
-        <v>12:15</v>
+        <v>19:00</v>
       </c>
       <c r="D93" t="str">
-        <v>15:00</v>
+        <v>21:45</v>
       </c>
       <c r="E93" t="str">
-        <v/>
+        <v>LSS-B (SG) / SCM-C (RK)</v>
       </c>
       <c r="F93" t="str">
-        <v>ABMBM (VPV)</v>
+        <v/>
       </c>
       <c r="G93" t="str">
         <v/>
       </c>
       <c r="H93" t="str">
-        <v/>
+        <v>DPI (SAA) / CCC (DS)</v>
       </c>
       <c r="I93" t="str">
         <v/>
@@ -6073,21 +6089,21 @@
         <v/>
       </c>
       <c r="L93" t="str">
-        <v>MTI-B (AK)</v>
+        <v/>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>2025-02-16</v>
+        <v>2025-03-01</v>
       </c>
       <c r="B94" t="str">
-        <v>Sunday</v>
+        <v>Saturday</v>
       </c>
       <c r="C94" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D94" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E94" t="str">
         <v/>
@@ -6096,16 +6112,16 @@
         <v/>
       </c>
       <c r="G94" t="str">
-        <v/>
+        <v>SAPM-B (VB) / AMA (PKB)</v>
       </c>
       <c r="H94" t="str">
         <v/>
       </c>
       <c r="I94" t="str">
-        <v>AIB-A (MPS) / CSP (SRA)</v>
+        <v/>
       </c>
       <c r="J94" t="str">
-        <v>SM (PB)</v>
+        <v/>
       </c>
       <c r="K94" t="str">
         <v/>
@@ -6116,19 +6132,19 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>2025-02-17</v>
+        <v>2025-03-02</v>
       </c>
       <c r="B95" t="str">
-        <v>Monday</v>
+        <v>Sunday</v>
       </c>
       <c r="C95" t="str">
-        <v>15:30</v>
+        <v>09:00</v>
       </c>
       <c r="D95" t="str">
-        <v>18:15</v>
+        <v>11:45</v>
       </c>
       <c r="E95" t="str">
-        <v/>
+        <v>LSS-B (SG)</v>
       </c>
       <c r="F95" t="str">
         <v/>
@@ -6143,7 +6159,7 @@
         <v/>
       </c>
       <c r="J95" t="str">
-        <v>MBM (JT)</v>
+        <v/>
       </c>
       <c r="K95" t="str">
         <v/>
@@ -6154,22 +6170,22 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>2025-02-18</v>
+        <v>2025-03-02</v>
       </c>
       <c r="B96" t="str">
-        <v>Tuesday</v>
+        <v>Sunday</v>
       </c>
       <c r="C96" t="str">
-        <v>19:00</v>
+        <v>12:15</v>
       </c>
       <c r="D96" t="str">
-        <v>21:45</v>
+        <v>15:00</v>
       </c>
       <c r="E96" t="str">
         <v/>
       </c>
       <c r="F96" t="str">
-        <v/>
+        <v>ABMBM (VPV)</v>
       </c>
       <c r="G96" t="str">
         <v/>
@@ -6178,7 +6194,7 @@
         <v/>
       </c>
       <c r="I96" t="str">
-        <v>AIB-B (VK)</v>
+        <v/>
       </c>
       <c r="J96" t="str">
         <v/>
@@ -6192,16 +6208,16 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>2025-02-19</v>
+        <v>2025-03-02</v>
       </c>
       <c r="B97" t="str">
-        <v>Wednesday</v>
+        <v>Sunday</v>
       </c>
       <c r="C97" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D97" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E97" t="str">
         <v/>
@@ -6210,13 +6226,13 @@
         <v/>
       </c>
       <c r="G97" t="str">
-        <v>SAPM-B (VB) / PF (PKB)</v>
+        <v/>
       </c>
       <c r="H97" t="str">
         <v/>
       </c>
       <c r="I97" t="str">
-        <v/>
+        <v>AIB-A (MPS)</v>
       </c>
       <c r="J97" t="str">
         <v/>
@@ -6230,16 +6246,16 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>2025-02-20</v>
+        <v>2025-03-03</v>
       </c>
       <c r="B98" t="str">
-        <v>Thursday</v>
+        <v>Monday</v>
       </c>
       <c r="C98" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D98" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E98" t="str">
         <v/>
@@ -6257,21 +6273,21 @@
         <v/>
       </c>
       <c r="J98" t="str">
-        <v/>
+        <v>PBM-A (JJ)</v>
       </c>
       <c r="K98" t="str">
         <v/>
       </c>
       <c r="L98" t="str">
-        <v>MTI-A (PV)</v>
+        <v/>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>2025-02-21</v>
+        <v>2025-03-04</v>
       </c>
       <c r="B99" t="str">
-        <v>Friday</v>
+        <v>Tuesday</v>
       </c>
       <c r="C99" t="str">
         <v>19:00</v>
@@ -6280,7 +6296,7 @@
         <v>21:45</v>
       </c>
       <c r="E99" t="str">
-        <v>SCM-A (ASS) / SCM-C (RK)</v>
+        <v/>
       </c>
       <c r="F99" t="str">
         <v/>
@@ -6289,10 +6305,10 @@
         <v/>
       </c>
       <c r="H99" t="str">
-        <v>ACCTP (DS)</v>
+        <v/>
       </c>
       <c r="I99" t="str">
-        <v/>
+        <v>CSP (SRA)</v>
       </c>
       <c r="J99" t="str">
         <v/>
@@ -6306,10 +6322,10 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>2025-02-22</v>
+        <v>2025-03-06</v>
       </c>
       <c r="B100" t="str">
-        <v>Saturday</v>
+        <v>Thursday</v>
       </c>
       <c r="C100" t="str">
         <v>19:00</v>
@@ -6321,10 +6337,10 @@
         <v/>
       </c>
       <c r="F100" t="str">
-        <v/>
+        <v>GT (AG)</v>
       </c>
       <c r="G100" t="str">
-        <v>SAPM-B (VB) / PF (PKB)</v>
+        <v/>
       </c>
       <c r="H100" t="str">
         <v/>
@@ -6344,19 +6360,19 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>2025-02-23</v>
+        <v>2025-03-07</v>
       </c>
       <c r="B101" t="str">
-        <v>Sunday</v>
+        <v>Friday</v>
       </c>
       <c r="C101" t="str">
-        <v>09:00</v>
+        <v>19:00</v>
       </c>
       <c r="D101" t="str">
-        <v>11:45</v>
+        <v>21:45</v>
       </c>
       <c r="E101" t="str">
-        <v>SCM-A (ASS) / SCM-C (RK)</v>
+        <v>SCM-C (RK)</v>
       </c>
       <c r="F101" t="str">
         <v/>
@@ -6365,7 +6381,7 @@
         <v/>
       </c>
       <c r="H101" t="str">
-        <v>ACCTP (DS)</v>
+        <v>DPI (SAA) / CCC (DS)</v>
       </c>
       <c r="I101" t="str">
         <v/>
@@ -6382,19 +6398,19 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>2025-02-23</v>
+        <v>2025-03-09</v>
       </c>
       <c r="B102" t="str">
         <v>Sunday</v>
       </c>
       <c r="C102" t="str">
-        <v>12:15</v>
+        <v>09:00</v>
       </c>
       <c r="D102" t="str">
-        <v>15:00</v>
+        <v>11:45</v>
       </c>
       <c r="E102" t="str">
-        <v/>
+        <v>SCM-B (SSP) / SCM-A (ASS) / LSS-A (GN)</v>
       </c>
       <c r="F102" t="str">
         <v/>
@@ -6415,21 +6431,21 @@
         <v/>
       </c>
       <c r="L102" t="str">
-        <v>MTI-A (PV)</v>
+        <v/>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>2025-02-23</v>
+        <v>2025-03-09</v>
       </c>
       <c r="B103" t="str">
         <v>Sunday</v>
       </c>
       <c r="C103" t="str">
-        <v>15:30</v>
+        <v>12:15</v>
       </c>
       <c r="D103" t="str">
-        <v>18:15</v>
+        <v>15:00</v>
       </c>
       <c r="E103" t="str">
         <v/>
@@ -6444,24 +6460,24 @@
         <v/>
       </c>
       <c r="I103" t="str">
-        <v>AIB-B (VK)</v>
+        <v/>
       </c>
       <c r="J103" t="str">
-        <v>MBM (JT)</v>
+        <v/>
       </c>
       <c r="K103" t="str">
         <v/>
       </c>
       <c r="L103" t="str">
-        <v/>
+        <v>SI-B (PV) / MASA (KKS) / SI-A (AK)</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>2025-02-24</v>
+        <v>2025-03-09</v>
       </c>
       <c r="B104" t="str">
-        <v>Monday</v>
+        <v>Sunday</v>
       </c>
       <c r="C104" t="str">
         <v>15:30</v>
@@ -6482,10 +6498,10 @@
         <v/>
       </c>
       <c r="I104" t="str">
-        <v/>
+        <v>AIB-B (VK)</v>
       </c>
       <c r="J104" t="str">
-        <v>SM (PB) / PBM-A (JJ) / PBM-B (SS)</v>
+        <v>PBM-A (JJ) / MMT (PN) / PBM-B (SS)</v>
       </c>
       <c r="K104" t="str">
         <v/>
@@ -6496,10 +6512,10 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>2025-02-26</v>
+        <v>2025-03-13</v>
       </c>
       <c r="B105" t="str">
-        <v>Wednesday</v>
+        <v>Thursday</v>
       </c>
       <c r="C105" t="str">
         <v>19:00</v>
@@ -6511,10 +6527,10 @@
         <v/>
       </c>
       <c r="F105" t="str">
-        <v/>
+        <v>ABMBM (VPV) / IPP (SRN)</v>
       </c>
       <c r="G105" t="str">
-        <v>PF (PKB) / ACF (ARS)</v>
+        <v/>
       </c>
       <c r="H105" t="str">
         <v/>
@@ -6526,7 +6542,7 @@
         <v/>
       </c>
       <c r="K105" t="str">
-        <v>LSO (PNR)</v>
+        <v/>
       </c>
       <c r="L105" t="str">
         <v/>
@@ -6534,10 +6550,10 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>2025-02-27</v>
+        <v>2025-03-14</v>
       </c>
       <c r="B106" t="str">
-        <v>Thursday</v>
+        <v>Friday</v>
       </c>
       <c r="C106" t="str">
         <v>19:00</v>
@@ -6546,16 +6562,16 @@
         <v>21:45</v>
       </c>
       <c r="E106" t="str">
-        <v/>
+        <v>LSS-A (GN) / LSS-B (SG)</v>
       </c>
       <c r="F106" t="str">
-        <v>GT (AG) / IPP (SRN)</v>
+        <v/>
       </c>
       <c r="G106" t="str">
         <v/>
       </c>
       <c r="H106" t="str">
-        <v/>
+        <v>ACCTP (DS)</v>
       </c>
       <c r="I106" t="str">
         <v/>
@@ -6572,28 +6588,28 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>2025-02-28</v>
+        <v>2025-03-16</v>
       </c>
       <c r="B107" t="str">
-        <v>Friday</v>
+        <v>Sunday</v>
       </c>
       <c r="C107" t="str">
-        <v>19:00</v>
+        <v>12:15</v>
       </c>
       <c r="D107" t="str">
-        <v>21:45</v>
+        <v>15:00</v>
       </c>
       <c r="E107" t="str">
-        <v>SCM-A (ASS) / SCM-C (RK)</v>
+        <v/>
       </c>
       <c r="F107" t="str">
-        <v/>
+        <v>ABMBM (VPV) / GT (AG)</v>
       </c>
       <c r="G107" t="str">
         <v/>
       </c>
       <c r="H107" t="str">
-        <v>CCC (DS)</v>
+        <v/>
       </c>
       <c r="I107" t="str">
         <v/>
@@ -6610,16 +6626,16 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>2025-03-01</v>
+        <v>2025-03-16</v>
       </c>
       <c r="B108" t="str">
-        <v>Saturday</v>
+        <v>Sunday</v>
       </c>
       <c r="C108" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D108" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E108" t="str">
         <v/>
@@ -6628,13 +6644,13 @@
         <v/>
       </c>
       <c r="G108" t="str">
-        <v>PF (PKB) / ACF (ARS)</v>
+        <v/>
       </c>
       <c r="H108" t="str">
         <v/>
       </c>
       <c r="I108" t="str">
-        <v/>
+        <v>CSP (SRA) / AIB-A (MPS)</v>
       </c>
       <c r="J108" t="str">
         <v/>
@@ -6648,28 +6664,28 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>2025-03-02</v>
+        <v>2025-03-20</v>
       </c>
       <c r="B109" t="str">
-        <v>Sunday</v>
+        <v>Thursday</v>
       </c>
       <c r="C109" t="str">
-        <v>09:00</v>
+        <v>19:00</v>
       </c>
       <c r="D109" t="str">
-        <v>11:45</v>
+        <v>21:45</v>
       </c>
       <c r="E109" t="str">
-        <v>SCM-A (ASS) / SCM-C (RK)</v>
+        <v/>
       </c>
       <c r="F109" t="str">
-        <v/>
+        <v>IPP (SRN)</v>
       </c>
       <c r="G109" t="str">
         <v/>
       </c>
       <c r="H109" t="str">
-        <v>CCC (DS)</v>
+        <v/>
       </c>
       <c r="I109" t="str">
         <v/>
@@ -6681,33 +6697,33 @@
         <v/>
       </c>
       <c r="L109" t="str">
-        <v/>
+        <v>MTI-A (PV) / MTI-B (AK)</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>2025-03-02</v>
+        <v>2025-03-21</v>
       </c>
       <c r="B110" t="str">
-        <v>Sunday</v>
+        <v>Friday</v>
       </c>
       <c r="C110" t="str">
-        <v>12:15</v>
+        <v>19:00</v>
       </c>
       <c r="D110" t="str">
-        <v>15:00</v>
+        <v>21:45</v>
       </c>
       <c r="E110" t="str">
         <v/>
       </c>
       <c r="F110" t="str">
-        <v>GT (AG) / IPP (SRN)</v>
+        <v/>
       </c>
       <c r="G110" t="str">
         <v/>
       </c>
       <c r="H110" t="str">
-        <v/>
+        <v>CCC (DS)</v>
       </c>
       <c r="I110" t="str">
         <v/>
@@ -6724,7 +6740,7 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>2025-03-02</v>
+        <v>2025-03-23</v>
       </c>
       <c r="B111" t="str">
         <v>Sunday</v>
@@ -6748,10 +6764,10 @@
         <v/>
       </c>
       <c r="I111" t="str">
-        <v/>
+        <v>AIB-B (VK)</v>
       </c>
       <c r="J111" t="str">
-        <v>SM (PB) / PBM-A (JJ) / PBM-B (SS)</v>
+        <v/>
       </c>
       <c r="K111" t="str">
         <v/>
@@ -6762,16 +6778,16 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>2025-03-03</v>
+        <v>2025-03-28</v>
       </c>
       <c r="B112" t="str">
-        <v>Monday</v>
+        <v>Friday</v>
       </c>
       <c r="C112" t="str">
-        <v>15:30</v>
+        <v>19:00</v>
       </c>
       <c r="D112" t="str">
-        <v>18:15</v>
+        <v>21:45</v>
       </c>
       <c r="E112" t="str">
         <v/>
@@ -6783,13 +6799,13 @@
         <v/>
       </c>
       <c r="H112" t="str">
-        <v/>
+        <v>ACCTP (DS)</v>
       </c>
       <c r="I112" t="str">
         <v/>
       </c>
       <c r="J112" t="str">
-        <v>PBM-B (SS) / MMT (PN) / UOSWTPB (PS)</v>
+        <v/>
       </c>
       <c r="K112" t="str">
         <v/>
@@ -6800,16 +6816,16 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>2025-03-04</v>
+        <v>2025-03-30</v>
       </c>
       <c r="B113" t="str">
-        <v>Tuesday</v>
+        <v>Sunday</v>
       </c>
       <c r="C113" t="str">
-        <v>19:00</v>
+        <v>15:30</v>
       </c>
       <c r="D113" t="str">
-        <v>21:45</v>
+        <v>18:15</v>
       </c>
       <c r="E113" t="str">
         <v/>
@@ -6824,7 +6840,7 @@
         <v/>
       </c>
       <c r="I113" t="str">
-        <v>CSP (SRA)</v>
+        <v>CSP (SRA) / AIB-A (MPS)</v>
       </c>
       <c r="J113" t="str">
         <v/>
@@ -6838,10 +6854,10 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>2025-03-06</v>
+        <v>2025-04-04</v>
       </c>
       <c r="B114" t="str">
-        <v>Thursday</v>
+        <v>Friday</v>
       </c>
       <c r="C114" t="str">
         <v>19:00</v>
@@ -6853,13 +6869,13 @@
         <v/>
       </c>
       <c r="F114" t="str">
-        <v>GT (AG)</v>
+        <v/>
       </c>
       <c r="G114" t="str">
         <v/>
       </c>
       <c r="H114" t="str">
-        <v/>
+        <v>CCC (DS) / DPI (SAA)</v>
       </c>
       <c r="I114" t="str">
         <v/>
@@ -6871,463 +6887,56 @@
         <v/>
       </c>
       <c r="L114" t="str">
-        <v>MTI-A (PV)</v>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="str">
-        <v>2025-03-07</v>
-      </c>
-      <c r="B115" t="str">
-        <v>Friday</v>
-      </c>
-      <c r="C115" t="str">
-        <v>19:00</v>
-      </c>
-      <c r="D115" t="str">
-        <v>21:45</v>
-      </c>
-      <c r="E115" t="str">
-        <v>SCM-A (ASS) / LSS-A (GN) / LSS-B (SG)</v>
-      </c>
-      <c r="F115" t="str">
-        <v/>
-      </c>
-      <c r="G115" t="str">
-        <v/>
-      </c>
-      <c r="H115" t="str">
-        <v/>
-      </c>
-      <c r="I115" t="str">
-        <v/>
-      </c>
-      <c r="J115" t="str">
-        <v/>
-      </c>
-      <c r="K115" t="str">
-        <v/>
-      </c>
-      <c r="L115" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="str">
-        <v>2025-03-09</v>
-      </c>
-      <c r="B116" t="str">
-        <v>Sunday</v>
-      </c>
-      <c r="C116" t="str">
-        <v>09:00</v>
-      </c>
-      <c r="D116" t="str">
-        <v>11:45</v>
-      </c>
-      <c r="E116" t="str">
-        <v>SCM-A (ASS) / LSS-A (GN) / LSS-B (SG)</v>
-      </c>
-      <c r="F116" t="str">
-        <v/>
-      </c>
-      <c r="G116" t="str">
-        <v/>
-      </c>
-      <c r="H116" t="str">
-        <v/>
-      </c>
-      <c r="I116" t="str">
-        <v/>
-      </c>
-      <c r="J116" t="str">
-        <v/>
-      </c>
-      <c r="K116" t="str">
-        <v/>
-      </c>
-      <c r="L116" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="str">
-        <v>2025-03-09</v>
-      </c>
-      <c r="B117" t="str">
-        <v>Sunday</v>
-      </c>
-      <c r="C117" t="str">
-        <v>12:15</v>
-      </c>
-      <c r="D117" t="str">
-        <v>15:00</v>
-      </c>
-      <c r="E117" t="str">
-        <v/>
-      </c>
-      <c r="F117" t="str">
-        <v>GT (AG)</v>
-      </c>
-      <c r="G117" t="str">
-        <v/>
-      </c>
-      <c r="H117" t="str">
-        <v/>
-      </c>
-      <c r="I117" t="str">
-        <v/>
-      </c>
-      <c r="J117" t="str">
-        <v/>
-      </c>
-      <c r="K117" t="str">
-        <v/>
-      </c>
-      <c r="L117" t="str">
-        <v>MTI-A (PV)</v>
+        <v/>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>2025-03-09</v>
+        <v>__META__</v>
       </c>
       <c r="B118" t="str">
-        <v>Sunday</v>
+        <v>Status</v>
       </c>
       <c r="C118" t="str">
-        <v>15:30</v>
-      </c>
-      <c r="D118" t="str">
-        <v>18:15</v>
-      </c>
-      <c r="E118" t="str">
-        <v/>
-      </c>
-      <c r="F118" t="str">
-        <v/>
-      </c>
-      <c r="G118" t="str">
-        <v/>
-      </c>
-      <c r="H118" t="str">
-        <v/>
-      </c>
-      <c r="I118" t="str">
-        <v>CSP (SRA)</v>
-      </c>
-      <c r="J118" t="str">
-        <v>PBM-B (SS) / MMT (PN) / UOSWTPB (PS)</v>
-      </c>
-      <c r="K118" t="str">
-        <v/>
-      </c>
-      <c r="L118" t="str">
-        <v/>
+        <v>Feasible</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>2025-03-13</v>
+        <v>__META__</v>
       </c>
       <c r="B119" t="str">
-        <v>Thursday</v>
+        <v>Generated At</v>
       </c>
       <c r="C119" t="str">
-        <v>19:00</v>
-      </c>
-      <c r="D119" t="str">
-        <v>21:45</v>
-      </c>
-      <c r="E119" t="str">
-        <v/>
-      </c>
-      <c r="F119" t="str">
-        <v/>
-      </c>
-      <c r="G119" t="str">
-        <v/>
-      </c>
-      <c r="H119" t="str">
-        <v/>
-      </c>
-      <c r="I119" t="str">
-        <v/>
-      </c>
-      <c r="J119" t="str">
-        <v/>
-      </c>
-      <c r="K119" t="str">
-        <v/>
-      </c>
-      <c r="L119" t="str">
-        <v>SI-B (PV)</v>
+        <v>2026-06-26T16:44:46.954Z</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>2025-03-14</v>
+        <v>__META__</v>
       </c>
       <c r="B120" t="str">
-        <v>Friday</v>
+        <v>Constraint</v>
       </c>
       <c r="C120" t="str">
-        <v>19:00</v>
-      </c>
-      <c r="D120" t="str">
-        <v>21:45</v>
-      </c>
-      <c r="E120" t="str">
-        <v/>
-      </c>
-      <c r="F120" t="str">
-        <v/>
-      </c>
-      <c r="G120" t="str">
-        <v/>
-      </c>
-      <c r="H120" t="str">
-        <v>CCC (DS)</v>
-      </c>
-      <c r="I120" t="str">
-        <v/>
-      </c>
-      <c r="J120" t="str">
-        <v/>
-      </c>
-      <c r="K120" t="str">
-        <v/>
-      </c>
-      <c r="L120" t="str">
-        <v/>
+        <v>soft</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>2025-03-16</v>
+        <v>__META__</v>
       </c>
       <c r="B121" t="str">
-        <v>Sunday</v>
-      </c>
-      <c r="C121" t="str">
-        <v>09:00</v>
-      </c>
-      <c r="D121" t="str">
-        <v>11:45</v>
-      </c>
-      <c r="E121" t="str">
-        <v/>
-      </c>
-      <c r="F121" t="str">
-        <v/>
-      </c>
-      <c r="G121" t="str">
-        <v/>
-      </c>
-      <c r="H121" t="str">
-        <v>CCC (DS)</v>
-      </c>
-      <c r="I121" t="str">
-        <v/>
-      </c>
-      <c r="J121" t="str">
-        <v/>
-      </c>
-      <c r="K121" t="str">
-        <v/>
-      </c>
-      <c r="L121" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="str">
-        <v>2025-03-16</v>
-      </c>
-      <c r="B122" t="str">
-        <v>Sunday</v>
-      </c>
-      <c r="C122" t="str">
-        <v>12:15</v>
-      </c>
-      <c r="D122" t="str">
-        <v>15:00</v>
-      </c>
-      <c r="E122" t="str">
-        <v/>
-      </c>
-      <c r="F122" t="str">
-        <v/>
-      </c>
-      <c r="G122" t="str">
-        <v/>
-      </c>
-      <c r="H122" t="str">
-        <v/>
-      </c>
-      <c r="I122" t="str">
-        <v/>
-      </c>
-      <c r="J122" t="str">
-        <v/>
-      </c>
-      <c r="K122" t="str">
-        <v/>
-      </c>
-      <c r="L122" t="str">
-        <v>SI-B (PV)</v>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="str">
-        <v>2025-03-21</v>
-      </c>
-      <c r="B123" t="str">
-        <v>Friday</v>
-      </c>
-      <c r="C123" t="str">
-        <v>19:00</v>
-      </c>
-      <c r="D123" t="str">
-        <v>21:45</v>
-      </c>
-      <c r="E123" t="str">
-        <v/>
-      </c>
-      <c r="F123" t="str">
-        <v/>
-      </c>
-      <c r="G123" t="str">
-        <v/>
-      </c>
-      <c r="H123" t="str">
-        <v>ACCTP (DS)</v>
-      </c>
-      <c r="I123" t="str">
-        <v/>
-      </c>
-      <c r="J123" t="str">
-        <v/>
-      </c>
-      <c r="K123" t="str">
-        <v/>
-      </c>
-      <c r="L123" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="str">
-        <v>2025-03-23</v>
-      </c>
-      <c r="B124" t="str">
-        <v>Sunday</v>
-      </c>
-      <c r="C124" t="str">
-        <v>15:30</v>
-      </c>
-      <c r="D124" t="str">
-        <v>18:15</v>
-      </c>
-      <c r="E124" t="str">
-        <v/>
-      </c>
-      <c r="F124" t="str">
-        <v/>
-      </c>
-      <c r="G124" t="str">
-        <v/>
-      </c>
-      <c r="H124" t="str">
-        <v/>
-      </c>
-      <c r="I124" t="str">
-        <v>AIB-B (VK)</v>
-      </c>
-      <c r="J124" t="str">
-        <v/>
-      </c>
-      <c r="K124" t="str">
-        <v/>
-      </c>
-      <c r="L124" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="str">
-        <v>2025-04-04</v>
-      </c>
-      <c r="B125" t="str">
-        <v>Friday</v>
-      </c>
-      <c r="C125" t="str">
-        <v>19:00</v>
-      </c>
-      <c r="D125" t="str">
-        <v>21:45</v>
-      </c>
-      <c r="E125" t="str">
-        <v/>
-      </c>
-      <c r="F125" t="str">
-        <v/>
-      </c>
-      <c r="G125" t="str">
-        <v/>
-      </c>
-      <c r="H125" t="str">
-        <v>ACCTP (DS) / DPI (SAA)</v>
-      </c>
-      <c r="I125" t="str">
-        <v/>
-      </c>
-      <c r="J125" t="str">
-        <v/>
-      </c>
-      <c r="K125" t="str">
-        <v/>
-      </c>
-      <c r="L125" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="str">
-        <v>__META__</v>
-      </c>
-      <c r="B129" t="str">
-        <v>Generated At</v>
-      </c>
-      <c r="C129" t="str">
-        <v>2026-06-06T21:32:37.345551</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="str">
-        <v>__META__</v>
-      </c>
-      <c r="B130" t="str">
-        <v>Constraint</v>
-      </c>
-      <c r="C130" t="str">
-        <v>soft</v>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="str">
-        <v>__META__</v>
-      </c>
-      <c r="B131" t="str">
         <v>Penalty</v>
       </c>
-      <c r="C131">
-        <v>0</v>
+      <c r="C121">
+        <v>0.3</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L131"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L121"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>